<commit_message>
Assumption M by exact quadrature, K>=2 chain, box cost, minimax lower bound, note cleanup, LaTeX update
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1028,7 +1028,7 @@
       </c>
       <c r="M6" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196).</t>
+          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled).</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="M15" s="33" t="inlineStr">
         <is>
-          <t>DECISION 2026-10-25: bounded variation as piecewise-Lipschitz class (Lipschitz rate Delta, &lt;=J jumps of size &lt;=D, box mu_t in [mu,c_mu*mu], eps_t in [eps,c_eps*eps], fixed reference Fisher norm). Target for P13: eta*sigma^2 + Delta^2/eta^2 (response of a time-varying-gain filter, gain eta*mu_t/eps) + J*D^2/(eta*T); sigma^2=r/(2*eff) (K=1 alpha known: mu/(2*eps*m)). Verified numerically (causal sampling): sinusoid, triangle, ramp, random walk, jumps; K=1,2,3 (grids (1,2),(1,4),(1,2,4),(1,3,9)); noise coeff r/(2 eff) within 3-13% in window; linear window eta&lt;=theta_k*mu^2/a, theta_k~0.013-0.03 (k-dependent). Problem 5 recursion verbatim cannot track drift (needs forgetting). RETRACTED c_lag~1.8: extra lag for alpha-unknown is an amplitude effect of the data-driven preconditioner (1.3-1.75x at A=0.2-0.5, -&gt;1 as A-&gt;0), absent with fixed preconditioner. Metric equivalence kappa_I: K=1 7-9, K=2 10-11 (mu x1.5), eps-independent. Hall-Willett VERIFIED (adversarial regret, no parameter-drift model). Solo (Piggott-Solo ICASSP 2018) NOT read: closed access, no OA copy (needs your library). Open: K&gt;=4, eps&lt;0.4 for K&gt;=2, analytic derivation of the adaptive-preconditioner excess. See problem14_drift_model.md</t>
+          <t>DECISION 2026-10-25: bounded variation as piecewise-Lipschitz class (Lipschitz rate Delta, &lt;=J jumps of size &lt;=D, box mu_t in [mu,c_mu*mu], eps_t in [eps,c_eps*eps], fixed reference Fisher norm). Target for P13: eta*sigma^2 + Delta^2/eta^2 (response of a time-varying-gain filter, gain eta*mu_t/eps) + J*D^2/(eta*T); sigma^2=r/(2*eff) (K=1 alpha known: mu/(2*eps*m)). Verified numerically (causal sampling): sinusoid, triangle, ramp, random walk, jumps; K=1,2,3 (grids (1,2),(1,4),(1,2,4),(1,3,9)); noise coeff r/(2 eff) within 3-13% in window; linear window eta&lt;=theta_k*mu^2/a, theta_k~0.013-0.03 (k-dependent). Problem 5 recursion verbatim cannot track drift (needs forgetting). RETRACTED c_lag~1.8: extra lag for alpha-unknown is an amplitude effect of the data-driven preconditioner (1.3-1.75x at A=0.2-0.5, -&gt;1 as A-&gt;0), absent with fixed preconditioner. Metric equivalence kappa_I: K=1 7-9, K=2 10-11 (mu x1.5), eps-independent. Hall-Willett VERIFIED from LaTeX source (adversarial regret C(1+sum||lam_{t+1}-Phi_t(lam_t)||_2)*sqrt(T): variation measure is a path length relative to known dynamics, norm not squared; no parameter-drift model). Solo (Piggott-Solo ICASSP 2018) NOT read: closed access, no OA copy (needs your library). Open: K&gt;=4, eps&lt;0.4 for K&gt;=2, analytic derivation of the adaptive-preconditioner excess. See problem14_drift_model.md CLEANUP 25 Oct: stale c_lag / amplitude-independence / K=2 bias-ratio statements struck in the note; noise convention (sigma^2=a=r/(2 eff)); path-length bound V^2/(eta T) (factor 1/2 not derived); jump term units. Label clashes resolved in LABELS.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Close problems 2, 4, 5, 7: closed-form lambda_min chain, dense F-norm projection, Theorem HP, Lemma JD
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -844,12 +844,12 @@
       </c>
       <c r="L3" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M3" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem02_identifiability.md; code/p2_window_bound.py, p2_lemma3_check.py, p2_gram_bound.py, p2_truncation_check.py, p2_truncation_bound.py. Fixed a thinning bug in p2_identifiability.py (had made lam_min ~10x too small for K&gt;=2). Findings (mu=1, beta=r^(k-1), MC 60-80k events): K&gt;=2 lam_min does NOT shrink with eps (K=2: ~0.045 at r=2, ~0.065 at r=4), cond ~ 1/eps (K=1: eps^-2); lam_min falls ~10x per added exponential (r=2: 0.069, 0.046, 0.0045 for K=1,2,3 at eps=0.1). Lower bounds: (1) Gram-matrix route is rigorous but useless (1e-6 to 1e-16 of truth, decays like eps^(2K+1)). (2) Theorem T (truncation + Lemma-B moments): lam_min(I) &gt;= (1/L)[lam_min(M) - sqrt(E|a|^4) sqrt(E lam^p / L^p)], M = E[a a^T] exact via a K^2 linear system (matches MC to 1-3%); bound is 2e-3 to 5e-2 of the MC lam_min for K&lt;=3 and non-vacuous; pure truncation without tail penalty would be within 2-8x. Open: closed-form formula in K and grid ratio, sharper tail bound, eps-sharpness for K&gt;=2. Depends on Lemma B (Problem 3 draft). Draft, not independently verified.</t>
+          <t>25 Oct 2026. problem02_identifiability.md; code/p2_window_bound.py, p2_lemma3_check.py, p2_gram_bound.py, p2_truncation_check.py, p2_truncation_bound.py. Fixed a thinning bug in p2_identifiability.py (had made lam_min ~10x too small for K&gt;=2). Findings (mu=1, beta=r^(k-1), MC 60-80k events): K&gt;=2 lam_min does NOT shrink with eps (K=2: ~0.045 at r=2, ~0.065 at r=4), cond ~ 1/eps (K=1: eps^-2); lam_min falls ~10x per added exponential (r=2: 0.069, 0.046, 0.0045 for K=1,2,3 at eps=0.1). Lower bounds: (1) Gram-matrix route is rigorous but useless (1e-6 to 1e-16 of truth, decays like eps^(2K+1)). (2) Theorem T (truncation + Lemma-B moments): lam_min(I) &gt;= (1/L)[lam_min(M) - sqrt(E|a|^4) sqrt(E lam^p / L^p)], M = E[a a^T] exact via a K^2 linear system (matches MC to 1-3%); bound is 2e-3 to 5e-2 of the MC lam_min for K&lt;=3 and non-vacuous; pure truncation without tail penalty would be within 2-8x. Open: closed-form formula in K and grid ratio, sharper tail bound, eps-sharpness for K&gt;=2. Depends on Lemma B (Problem 3 draft). Draft, not independently verified. CLOSED 25 Oct (Done): closed-form chain in K and grid ratio r: Cov(S) &gt;= (E lam/4) G (G=1/(b_i+b_j), spectral), exact E S_k = mu/(eps b_k), lam_min(M) &gt;= lam_min(C)/(1+2|m|^2), Cauchy inverse in closed form, then truncation with Lemma-1' moments; valid but 1e3-1e8 below truth (code/p2_closed_chain.py). Sharp scaling = three-tier structure (Problem 12), heuristic.</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="L5" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M5" s="33" t="inlineStr">
         <is>
-          <t>24-25 Oct 2026. problem04_projection.md, code/p4_projection.py. Exact projection onto {mu&gt;=mu_min, alpha&gt;=0, sum alpha_k/beta_k&lt;=1-eps} in a DIAGONAL metric: mu separable; alpha_k = max(0, y_k - tau*w_k/d_k), tau from sorted breakpoints, O(K log K); matches SLSQP on 300 random instances (4e-6); &lt;1 ms for K up to 1e4. Regret-constant effect: non-expansive in the update's own metric, so no extra constant; the cost is cond(D^-1/2 I D^-1/2). K=1: universal ~5.83 (rho^2-&gt;1/2), independent of eps (raw ~1e6 at eps=1e-3). K&gt;=2 (corrected 25 Oct after fixing a simulator bug): scaled cond only 1.2-3x below raw and still grows as eps falls (K=2,r=2: 118-&gt;368; K=3: 765-&gt;2477), so a diagonal metric is NOT enough for K&gt;=2. Open: dense-metric projection (QP, ~O(K^2)), O(K) version, K&gt;=2 preconditioner. Status In progress because 'Done when' asks for the Fisher/ONS metric. UPDATE 25 Oct (problem05_circularity.md): for K=1 the diagonal clip is NOT adequate: it violates non-expansiveness in 0.7-4.6% of steps and inflates regret ~10x when the box is tight (E R_n 16 vs 3.5 at eps=.1; 79 vs 5.4 at eps=.03). Exact F-norm projection onto a box is O(1) for K=1 (edge minimisers + corners) and had 0 violations in 24 configs. Use it.</t>
+          <t>24-25 Oct 2026. problem04_projection.md, code/p4_projection.py. Exact projection onto {mu&gt;=mu_min, alpha&gt;=0, sum alpha_k/beta_k&lt;=1-eps} in a DIAGONAL metric: mu separable; alpha_k = max(0, y_k - tau*w_k/d_k), tau from sorted breakpoints, O(K log K); matches SLSQP on 300 random instances (4e-6); &lt;1 ms for K up to 1e4. Regret-constant effect: non-expansive in the update's own metric, so no extra constant; the cost is cond(D^-1/2 I D^-1/2). K=1: universal ~5.83 (rho^2-&gt;1/2), independent of eps (raw ~1e6 at eps=1e-3). K&gt;=2 (corrected 25 Oct after fixing a simulator bug): scaled cond only 1.2-3x below raw and still grows as eps falls (K=2,r=2: 118-&gt;368; K=3: 765-&gt;2477), so a diagonal metric is NOT enough for K&gt;=2. Open: dense-metric projection (QP, ~O(K^2)), O(K) version, K&gt;=2 preconditioner. Status In progress because 'Done when' asks for the Fisher/ONS metric. UPDATE 25 Oct (problem05_circularity.md): for K=1 the diagonal clip is NOT adequate: it violates non-expansiveness in 0.7-4.6% of steps and inflates regret ~10x when the box is tight (E R_n 16 vs 3.5 at eps=.1; 79 vs 5.4 at eps=.03). Exact F-norm projection onto a box is O(1) for K=1 (edge minimisers + corners) and had 0 violations in 24 configs. Use it. CLOSED 25 Oct (Done): dense F-norm projection for any K (BVLS + bisection on the budget multiplier): matches brute force to 5e-14, non-expansive (0 violations in 2000 pairs), O(K^3) per inner solve (19 ms K=2, 97 ms K=5); the diagonal O(K log K) algorithm remains for the diagonal metric (code/p4_dense_projection.py).</t>
         </is>
       </c>
     </row>
@@ -1023,12 +1023,12 @@
       </c>
       <c r="L6" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M6" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled).</t>
+          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled). CLOSED 25 Oct (Done): Theorem HP (problem05_07_closure.md): with prob &gt;= 1-6e^-x-P(E^c), R_n &lt;= psi_max(2 i0+3x) + 4[D0' + x/theta + G_n(x)]; plus expected-regret Thm R (sharp constant). Assumptions: known compact convex Theta_c, leverage event, Assumption M (certified K=1) / lambda_L (K&gt;=2).</t>
         </is>
       </c>
     </row>
@@ -1141,12 +1141,12 @@
       </c>
       <c r="L8" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M8" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem07_leverage.md; code/p5_leverage.py, p5_theorem_check.py, p5_component_check.py. K=1 only. Split gradient g = s (score at theta*) + h (drift). Lemma 7a (rigorous): E[s|past]=0, E[s s'|past]=E[dJ] (stopped martingale). Lemma 7b: E[h'F^-1 h] &lt;= (ell/mu_min) E[v'dF v], ell = sup_u phi'F^-1 phi/lam* (point leverage). Lemma 7c: tr(F^-1 dF) &lt;= r(x) logdet increment, r(x)=x/log(1+x) (gap leverage x). Theorem 7 (conditional on a.s. L1-L3): E R_n &lt;= [P0 + (1+eta) c+ r(x) E logdet(F_n/F_0)]/(1-B), B=(1+1/eta) ell/mu_min&lt;1, closing the gradient-norm term of Problem 5 (growth ~ d log T, constant ~3-6x too big). Leverage scale: worst case is the quiet gap, ell ~ [F^-1]_mumu/mu* ~ (k-1)/(eps T), so B&lt;1 needs ~4(k-1)/(eps^2 mu_min) events: leverage burn-in ~1/eps^2 events (matches Problem 3 mixing; observed medians 1520 at eps=.1, 10086 at eps=.03). Numerics: all three lemmas verified; drift term is negligible in practice (0.02 vs bound 3); full bound valid but 15-40x loose. NOT done: L1-L3 as stopping-time/high-probability statements (needs Fisher concentration, Problems 2-3), projection, K&gt;=2, sharp constant. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct: (L1) now holds by construction for the compact-box exact-projection algorithm (problem05_circularity.md); F &gt;= F0 + J/c+ verified PSD in all runs. Remaining: localisation bookkeeping. UPDATE 25 Oct: bootstrap done at polynomial-tail level (problem05_bootstrap.md); remaining for the leverage assumptions: exponential tails, localisation, K&gt;=2. UPDATE 25 Oct: exponential-tail versions of Theorem F and the bootstrap in problem05_exponential_tails.md (G_n control sketched only).</t>
+          <t>25 Oct 2026. problem07_leverage.md; code/p5_leverage.py, p5_theorem_check.py, p5_component_check.py. K=1 only. Split gradient g = s (score at theta*) + h (drift). Lemma 7a (rigorous): E[s|past]=0, E[s s'|past]=E[dJ] (stopped martingale). Lemma 7b: E[h'F^-1 h] &lt;= (ell/mu_min) E[v'dF v], ell = sup_u phi'F^-1 phi/lam* (point leverage). Lemma 7c: tr(F^-1 dF) &lt;= r(x) logdet increment, r(x)=x/log(1+x) (gap leverage x). Theorem 7 (conditional on a.s. L1-L3): E R_n &lt;= [P0 + (1+eta) c+ r(x) E logdet(F_n/F_0)]/(1-B), B=(1+1/eta) ell/mu_min&lt;1, closing the gradient-norm term of Problem 5 (growth ~ d log T, constant ~3-6x too big). Leverage scale: worst case is the quiet gap, ell ~ [F^-1]_mumu/mu* ~ (k-1)/(eps T), so B&lt;1 needs ~4(k-1)/(eps^2 mu_min) events: leverage burn-in ~1/eps^2 events (matches Problem 3 mixing; observed medians 1520 at eps=.1, 10086 at eps=.03). Numerics: all three lemmas verified; drift term is negligible in practice (0.02 vs bound 3); full bound valid but 15-40x loose. NOT done: L1-L3 as stopping-time/high-probability statements (needs Fisher concentration, Problems 2-3), projection, K&gt;=2, sharp constant. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct: (L1) now holds by construction for the compact-box exact-projection algorithm (problem05_circularity.md); F &gt;= F0 + J/c+ verified PSD in all runs. Remaining: localisation bookkeeping. UPDATE 25 Oct: bootstrap done at polynomial-tail level (problem05_bootstrap.md); remaining for the leverage assumptions: exponential tails, localisation, K&gt;=2. UPDATE 25 Oct: exponential-tail versions of Theorem F and the bootstrap in problem05_exponential_tails.md (G_n control sketched only). CLOSED 25 Oct (Done): Lemma JD (problem05_07_closure.md): joint zero mean and covariance E dJ (non-degenerate since b not parallel to a), pathwise |s|^2_{F^-1} &lt;= (2 lbar/mu)(1+E^2), tail e^-m, cumulative exponential bound (E5b); 0 violations in 1.44e6 gaps.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final audit: fix E5c constant, restate overstated impossibility, exact general-K identity, audit report
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1028,7 +1028,7 @@
       </c>
       <c r="M6" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled). CLOSED 25 Oct (Done): Theorem HP (problem05_07_closure.md): with prob &gt;= 1-6e^-x-P(E^c), R_n &lt;= psi_max(2 i0+3x) + 4[D0' + x/theta + G_n(x)]; plus expected-regret Thm R (sharp constant). Assumptions: known compact convex Theta_c, leverage event, Assumption M (certified K=1) / lambda_L (K&gt;=2).</t>
+          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled). CLOSED 25 Oct (Done): Theorem HP (problem05_07_closure.md): with prob &gt;= 1-6e^-x-P(E^c), R_n &lt;= psi_max(2 i0+3x) + 4[D0' + x/theta + G_n(x)]; plus expected-regret Thm R (sharp constant). Assumptions: known compact convex Theta_c, leverage event, Assumption M (certified K=1) / lambda_L (K&gt;=2). FINAL AUDIT 25 Oct (final_audit.md): fixed constant in Lemma E5c (xbar = lbar m/(c^- mu*), not c^+), replaced loose general-K Lemma E1 by the exact Z_c identity; K=2 pathwise Newton/martingale inequalities verified (code/p5_k2_pathwise_check.py).</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="M12" s="33" t="inlineStr">
         <is>
-          <t>Draft done 2026-10-25 (needs your re-derivation). DECISION: C4 uses STATIONARY observation, dichotomy = bounded vs divergent. Rigorous: K=1 full dichotomy (Thm A, B); ANY K with k_K=2*mu*sum(alpha/beta^2)/n: E[1/lam]=O(eps) if k_K&gt;1 (Thm E, corrected Lyapunov log W+psi/W^2 with Perron weights) =&gt; no consistent mu-estimator (Cor E'); E[1/lam]&gt;=c eps^(k_K+eta) if k_K&lt;1 (Thm F) =&gt; alpha-known information diverges. Pathwise check of generator bounds passed. Open: efficient (alpha-unknown) info divergence for K&gt;=2 (numerics eff/m-&gt;1), matching upper bound/estimator (MLE is mixed-normal: observed info random, CV~0.5), k_K=1 borderline, cold-start coefficients. See problem11_dichotomy.md LITERATURE 25 Oct: divergence of mu-information for kappa&lt;=1 is Herrera-Marin Remark 4.8 (Fatou); he states the kappa&gt;1 direction is NOT proved. Gamma shape/Feller threshold k=2*beta*mu/alpha^2 confirmed against Jaisson-Rosenbaum Thm 2.2 (shape 2m*mu; tested, autocorrelation exp(-eps*beta*t) also confirmed). REASSESSMENT 25 Oct: divergence half = Herrera-Marin Remark 4.8; he leaves the converse (kappa&gt;1) unproved. Other session's Theorem A (K=1, stationary) claims it with rates (I have NOT verified its proof). Exact slopes of (1/2) log det I vs log(1/eps): 0.347,0.397,0.404,0.403,0.402 -&gt; (1-k0)/2=0.40 for k0=0.2; -&gt; 0 for k0&gt;=2. K=2 dictionary: A_T matches the K=1 value at equal k=2*mu*m (1.29/1.53/1.79 vs 1.26/1.55/1.78): supports threshold 2*mu*sum(w_k/beta_k)=1. Observation model matters (stationary vs empty start). VERIFICATION 25 Oct (verification_thmA_E_F.md): Lemma H re-derived and holds pathwise in 30/30 (parameter,z) cases; Theorems E and F re-derived: CORRECT given Lemma H; E_pi[A f]=0 and the E/F integral inequalities confirmed by stationary MC (16 independent replicates). GAP in the use of E: Corollary E'/Theorem B compare path laws with the SAME initial state; impossibility is rigorous for the experiment where S_0 (pre-sample history) is given, but for a stationary record with unobserved past one also needs KL(pi_theta||pi_theta') = O(1) (Gamma approx 0.003-0.034; not proved) - same step Herrera-Marin I calls open. Also: the empty-start experiment (the actual streaming setting) has mu-information &gt;= ln T for every k, so the 'mu unlearnable' headline is observation-model specific. UPDATE 25 Oct (theoremA_step2_and_stationary_tv.md): initial-state gap closed for K=1, k0&gt;1: TV(Q,Q') &lt;= sqrt(rho u'I_T u/2) + TV(pi,pi') (Lemma R), and TV(pi_theta,pi_theta') &lt;= C|delta| + C eps^min(1,k0-1/2) via exact characteristic function phi=G*Ftilde (Gamma comparator), imaginary-axis bound |D_eps(-i tau)|&lt;=31.5/alpha, monotone |phi|, and TV &lt;= ||.||_H1/(2 sqrt2). Numerics (FFT inversion of exact ch.f.): TV(pi,pi') = 0.026/0.070 for delta=0.1/0.3, flat in eps from 0.1 to 0.003; TV(pi,Gamma) ~ eps. MY PROOF, NOT REVIEWED; constants not explicit; K&gt;=2, k0&lt;=1 not covered. UPDATE 25 Oct (general_K_impossibility.md): impossibility of consistent mu-estimation for the STATIONARY record with unobserved past now proved for ANY K with k_K&gt;1 (Theorem V: TV(Q,Q') &lt;= C delta sqrt(ln(1/delta))), by a route that bypasses TV(pi_theta,pi_theta'): (1) KL of stationary theta-process vs theta'-dynamics started from pi_theta over a window L+T=O(1/gamma) is O(delta^2) via Theorem E; (2) superposition: process from state s = empty-start + ghost immigrants g_s(t); (3) cluster survival q(s)&lt;=C' gamma e^{-gamma s} from the flow Y'=-BY+alpha(1-e^{-|Y|}) and zeta'=-gamma zeta - r(|Y|) (first-moment bound would lose ln(1/eps)). Verified: flow vs cluster MC (K=1,2), ghost-hit prob decays e^{-gamma L} (K=2 sim). MY PROOF, UNREVIEWED. TV(pi,pi') for K&gt;=2 itself still open. LITERATURE 25 Oct (literature_search_report.md): CIR side: information about the drift constant finite iff a &gt; sigma (Ben Alaya et al. Thm 2.1); MLE defined only for 2a &gt; sigma^2 (Dehtiar et al.); critical case sqrt(log T) rate. Discrete side: all estimation results found are CLSE/OLS; Li 2011: nonzero initial values =&gt; CLSE of immigration mean inconsistent; Anne-Lu-Yu-Zhou 2026: OLS intercept inconsistent in local-to-unity affine processes (no Hawkes, no information bound; overlap risk Medium). Herrera-Marin's Wei-Winnicki attribution UNVERIFIED. THM T CONSTANTS 25 Oct (thmT_explicit_constants.md): Theorem T now has an explicit chain: |d|&lt;=19 (true sup 1.143), tail exponent q=k0/(2(1+3/X0))&gt;1/2 (k/(1+r)^2=k0 exactly), certified TV(pi,Gamma)&lt;=Phi/(2 sqrt2); k0=2: 2e-2 (eps=1e-4), 1e-3 (1e-5), 8.6e-5 (1e-6); bound 1e2-1e3 above truth, valid in all tests. Ridge pair: TV&lt;=2.4e-3+0.39 delta (eps&lt;=1e-5, k0=2, delta&lt;=0.3). Phi by floating-point quadrature of hand-proved majorants, not interval arithmetic; KL step evaluated on a grid; informative only for eps&lt;~1e-4.</t>
+          <t>Draft done 2026-10-25 (needs your re-derivation). DECISION: C4 uses STATIONARY observation, dichotomy = bounded vs divergent. Rigorous: K=1 full dichotomy (Thm A, B); ANY K with k_K=2*mu*sum(alpha/beta^2)/n: E[1/lam]=O(eps) if k_K&gt;1 (Thm E, corrected Lyapunov log W+psi/W^2 with Perron weights) =&gt; no consistent mu-estimator (Cor E'); E[1/lam]&gt;=c eps^(k_K+eta) if k_K&lt;1 (Thm F) =&gt; alpha-known information diverges. Pathwise check of generator bounds passed. Open: efficient (alpha-unknown) info divergence for K&gt;=2 (numerics eff/m-&gt;1), matching upper bound/estimator (MLE is mixed-normal: observed info random, CV~0.5), k_K=1 borderline, cold-start coefficients. See problem11_dichotomy.md LITERATURE 25 Oct: divergence of mu-information for kappa&lt;=1 is Herrera-Marin Remark 4.8 (Fatou); he states the kappa&gt;1 direction is NOT proved. Gamma shape/Feller threshold k=2*beta*mu/alpha^2 confirmed against Jaisson-Rosenbaum Thm 2.2 (shape 2m*mu; tested, autocorrelation exp(-eps*beta*t) also confirmed). REASSESSMENT 25 Oct: divergence half = Herrera-Marin Remark 4.8; he leaves the converse (kappa&gt;1) unproved. Other session's Theorem A (K=1, stationary) claims it with rates (I have NOT verified its proof). Exact slopes of (1/2) log det I vs log(1/eps): 0.347,0.397,0.404,0.403,0.402 -&gt; (1-k0)/2=0.40 for k0=0.2; -&gt; 0 for k0&gt;=2. K=2 dictionary: A_T matches the K=1 value at equal k=2*mu*m (1.29/1.53/1.79 vs 1.26/1.55/1.78): supports threshold 2*mu*sum(w_k/beta_k)=1. Observation model matters (stationary vs empty start). VERIFICATION 25 Oct (verification_thmA_E_F.md): Lemma H re-derived and holds pathwise in 30/30 (parameter,z) cases; Theorems E and F re-derived: CORRECT given Lemma H; E_pi[A f]=0 and the E/F integral inequalities confirmed by stationary MC (16 independent replicates). GAP in the use of E: Corollary E'/Theorem B compare path laws with the SAME initial state; impossibility is rigorous for the experiment where S_0 (pre-sample history) is given, but for a stationary record with unobserved past one also needs KL(pi_theta||pi_theta') = O(1) (Gamma approx 0.003-0.034; not proved) - same step Herrera-Marin I calls open. Also: the empty-start experiment (the actual streaming setting) has mu-information &gt;= ln T for every k, so the 'mu unlearnable' headline is observation-model specific. UPDATE 25 Oct (theoremA_step2_and_stationary_tv.md): initial-state gap closed for K=1, k0&gt;1: TV(Q,Q') &lt;= sqrt(rho u'I_T u/2) + TV(pi,pi') (Lemma R), and TV(pi_theta,pi_theta') &lt;= C|delta| + C eps^min(1,k0-1/2) via exact characteristic function phi=G*Ftilde (Gamma comparator), imaginary-axis bound |D_eps(-i tau)|&lt;=31.5/alpha, monotone |phi|, and TV &lt;= ||.||_H1/(2 sqrt2). Numerics (FFT inversion of exact ch.f.): TV(pi,pi') = 0.026/0.070 for delta=0.1/0.3, flat in eps from 0.1 to 0.003; TV(pi,Gamma) ~ eps. MY PROOF, NOT REVIEWED; constants not explicit; K&gt;=2, k0&lt;=1 not covered. UPDATE 25 Oct (general_K_impossibility.md): impossibility of consistent mu-estimation for the STATIONARY record with unobserved past now proved for ANY K with k_K&gt;1 (Theorem V: TV(Q,Q') &lt;= C delta sqrt(ln(1/delta))), by a route that bypasses TV(pi_theta,pi_theta'): (1) KL of stationary theta-process vs theta'-dynamics started from pi_theta over a window L+T=O(1/gamma) is O(delta^2) via Theorem E; (2) superposition: process from state s = empty-start + ghost immigrants g_s(t); (3) cluster survival q(s)&lt;=C' gamma e^{-gamma s} from the flow Y'=-BY+alpha(1-e^{-|Y|}) and zeta'=-gamma zeta - r(|Y|) (first-moment bound would lose ln(1/eps)). Verified: flow vs cluster MC (K=1,2), ghost-hit prob decays e^{-gamma L} (K=2 sim). MY PROOF, UNREVIEWED. TV(pi,pi') for K&gt;=2 itself still open. LITERATURE 25 Oct (literature_search_report.md): CIR side: information about the drift constant finite iff a &gt; sigma (Ben Alaya et al. Thm 2.1); MLE defined only for 2a &gt; sigma^2 (Dehtiar et al.); critical case sqrt(log T) rate. Discrete side: all estimation results found are CLSE/OLS; Li 2011: nonzero initial values =&gt; CLSE of immigration mean inconsistent; Anne-Lu-Yu-Zhou 2026: OLS intercept inconsistent in local-to-unity affine processes (no Hawkes, no information bound; overlap risk Medium). Herrera-Marin's Wei-Winnicki attribution UNVERIFIED. THM T CONSTANTS 25 Oct (thmT_explicit_constants.md): Theorem T now has an explicit chain: |d|&lt;=19 (true sup 1.143), tail exponent q=k0/(2(1+3/X0))&gt;1/2 (k/(1+r)^2=k0 exactly), certified TV(pi,Gamma)&lt;=Phi/(2 sqrt2); k0=2: 2e-2 (eps=1e-4), 1e-3 (1e-5), 8.6e-5 (1e-6); bound 1e2-1e3 above truth, valid in all tests. Ridge pair: TV&lt;=2.4e-3+0.39 delta (eps&lt;=1e-5, k0=2, delta&lt;=0.3). Phi by floating-point quadrature of hand-proved majorants, not interval arithmetic; KL step evaluated on a grid; informative only for eps&lt;~1e-4. FINAL AUDIT 25 Oct (final_audit.md): the 'no consistent estimator given S0' statements (Thm B, Cor D, Cor E') were stronger than the KL lemma proves: the correct bound is TV(Q) &lt;= TV(pi_theta, pi_theta') + sqrt(rho T u'Iu/2). Rigorous impossibility: K=1 stationary record (Thm T), any K stationary record with unobserved past (Thm V). K&gt;=2 with S0 observed: open.</t>
         </is>
       </c>
     </row>
@@ -1613,10 +1613,14 @@
       </c>
       <c r="L16" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M16" s="33" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M16" s="33" t="inlineStr">
+        <is>
+          <t>Draft done 2026-10-25, CONDITIONAL on Problem 13 (tracking bound not proved; built on measured MSE structure from P14). MSE(eta)=a*eta+B(eta), a=r/(2*eff). Smooth drift fast regime: eta*=(Delta_e^2/a)^(1/3) ~ eps^(4/3)*Delta^(2/3) (k&gt;1), MSE*=1.5*a*eta*; jumps: eta*=D*mu/sqrt(2*a*L_e) ~ eps^(3/2); k&lt;1 exponents 1+k/3, 1+k/2. Window cap eta&lt;=theta*mu^2/a ~ eps^2 binds as eps-&gt;0. Tracking beats static estimator only if P*eff*(A*mu)^2 &gt;~ 16 (checked: 8.7 no gain, 22.6 modest, 34.7 gain 26%). alpha unknown shifts eta* down by ~k^(-1/3). Sim (K=1): smooth alpha-known eta_opt 0.00292/0.00179/0.00089 vs predicted 0.00295/0.00193/0.00095 at eps 0.4/0.3/0.2; jumps within 15-27%. Not done: K&gt;=2 eta_opt, eps&lt;0.2, pure power-law regime. See problem15_step_size.md</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="46.5" customHeight="1" s="27">
       <c r="A17" s="29" t="n">

</xml_diff>

<commit_message>
Strengthen: tangent-line minorant (sharp spectrum bounds, information level without Assumption M), complete proof of Theorem R
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -849,7 +849,7 @@
       </c>
       <c r="M3" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem02_identifiability.md; code/p2_window_bound.py, p2_lemma3_check.py, p2_gram_bound.py, p2_truncation_check.py, p2_truncation_bound.py. Fixed a thinning bug in p2_identifiability.py (had made lam_min ~10x too small for K&gt;=2). Findings (mu=1, beta=r^(k-1), MC 60-80k events): K&gt;=2 lam_min does NOT shrink with eps (K=2: ~0.045 at r=2, ~0.065 at r=4), cond ~ 1/eps (K=1: eps^-2); lam_min falls ~10x per added exponential (r=2: 0.069, 0.046, 0.0045 for K=1,2,3 at eps=0.1). Lower bounds: (1) Gram-matrix route is rigorous but useless (1e-6 to 1e-16 of truth, decays like eps^(2K+1)). (2) Theorem T (truncation + Lemma-B moments): lam_min(I) &gt;= (1/L)[lam_min(M) - sqrt(E|a|^4) sqrt(E lam^p / L^p)], M = E[a a^T] exact via a K^2 linear system (matches MC to 1-3%); bound is 2e-3 to 5e-2 of the MC lam_min for K&lt;=3 and non-vacuous; pure truncation without tail penalty would be within 2-8x. Open: closed-form formula in K and grid ratio, sharper tail bound, eps-sharpness for K&gt;=2. Depends on Lemma B (Problem 3 draft). Draft, not independently verified. CLOSED 25 Oct (Done): closed-form chain in K and grid ratio r: Cov(S) &gt;= (E lam/4) G (G=1/(b_i+b_j), spectral), exact E S_k = mu/(eps b_k), lam_min(M) &gt;= lam_min(C)/(1+2|m|^2), Cauchy inverse in closed form, then truncation with Lemma-1' moments; valid but 1e3-1e8 below truth (code/p2_closed_chain.py). Sharp scaling = three-tier structure (Problem 12), heuristic.</t>
+          <t>25 Oct 2026. problem02_identifiability.md; code/p2_window_bound.py, p2_lemma3_check.py, p2_gram_bound.py, p2_truncation_check.py, p2_truncation_bound.py. Fixed a thinning bug in p2_identifiability.py (had made lam_min ~10x too small for K&gt;=2). Findings (mu=1, beta=r^(k-1), MC 60-80k events): K&gt;=2 lam_min does NOT shrink with eps (K=2: ~0.045 at r=2, ~0.065 at r=4), cond ~ 1/eps (K=1: eps^-2); lam_min falls ~10x per added exponential (r=2: 0.069, 0.046, 0.0045 for K=1,2,3 at eps=0.1). Lower bounds: (1) Gram-matrix route is rigorous but useless (1e-6 to 1e-16 of truth, decays like eps^(2K+1)). (2) Theorem T (truncation + Lemma-B moments): lam_min(I) &gt;= (1/L)[lam_min(M) - sqrt(E|a|^4) sqrt(E lam^p / L^p)], M = E[a a^T] exact via a K^2 linear system (matches MC to 1-3%); bound is 2e-3 to 5e-2 of the MC lam_min for K&lt;=3 and non-vacuous; pure truncation without tail penalty would be within 2-8x. Open: closed-form formula in K and grid ratio, sharper tail bound, eps-sharpness for K&gt;=2. Depends on Lemma B (Problem 3 draft). Draft, not independently verified. CLOSED 25 Oct (Done): closed-form chain in K and grid ratio r: Cov(S) &gt;= (E lam/4) G (G=1/(b_i+b_j), spectral), exact E S_k = mu/(eps b_k), lam_min(M) &gt;= lam_min(C)/(1+2|m|^2), Cauchy inverse in closed form, then truncation with Lemma-1' moments; valid but 1e3-1e8 below truth (code/p2_closed_chain.py). Sharp scaling = three-tier structure (Problem 12), heuristic. STRENGTHENED 25 Oct (tangent_bound.md): tangent-line minorant I &gt;= (2/l0)M - (1/l0^2)M3 with exact moment systems (orders&lt;=3) gives a rigorous lower bound within 1.3-3.5x of Monte Carlo (K=1,2,3), correct eps-scaling (~0.25 eps); was 1e3-1e8 loose.</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="M6" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled). CLOSED 25 Oct (Done): Theorem HP (problem05_07_closure.md): with prob &gt;= 1-6e^-x-P(E^c), R_n &lt;= psi_max(2 i0+3x) + 4[D0' + x/theta + G_n(x)]; plus expected-regret Thm R (sharp constant). Assumptions: known compact convex Theta_c, leverage event, Assumption M (certified K=1) / lambda_L (K&gt;=2). FINAL AUDIT 25 Oct (final_audit.md): fixed constant in Lemma E5c (xbar = lbar m/(c^- mu*), not c^+), replaced loose general-K Lemma E1 by the exact Z_c identity; K=2 pathwise Newton/martingale inequalities verified (code/p5_k2_pathwise_check.py).</t>
+          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled). CLOSED 25 Oct (Done): Theorem HP (problem05_07_closure.md): with prob &gt;= 1-6e^-x-P(E^c), R_n &lt;= psi_max(2 i0+3x) + 4[D0' + x/theta + G_n(x)]; plus expected-regret Thm R (sharp constant). Assumptions: known compact convex Theta_c, leverage event, Assumption M (certified K=1) / lambda_L (K&gt;=2). FINAL AUDIT 25 Oct (final_audit.md): fixed constant in Lemma E5c (xbar = lbar m/(c^- mu*), not c^+), replaced loose general-K Lemma E1 by the exact Z_c identity; K=2 pathwise Newton/martingale inequalities verified (code/p5_k2_pathwise_check.py). STRENGTHENED 25 Oct: (1) theoremR_proof_complete.md writes every step of the expected-regret theorem (assembly needs only predictable good-gap indicators + one per-time failure bound H3); (2) information level without Assumption M via the tangent minorant: lambda_*/2 ~ 0.013 for the K=2 example vs ~1e-6 before.</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="M13" s="33" t="inlineStr">
         <is>
-          <t>Draft done 2026-10-25 (needs your re-derivation). I(theta*) has three tiers: top ~1/eps along grad_alpha n=(1/beta_k) (pure n-direction, best determined); K-1 middle 'kernel-shape' directions (sum w_k/beta_k=0) of size O(1) set by the beta-grid via the Hawkes-corrected spectral Gram (checked: 0.0667 pred vs 0.0661 MC, K=2); ridge ~ eps/(mu(k-1)) along (1,-eps*alpha/mu) = mean-rate-preserving mu-n trade (E lam=mu/eps fixed, shape fixed). As eps-&gt;0 the RIDGE is the degenerate direction; at moderate eps for K&gt;=3 / tight grids a time-scale MIXTURE is smaller (K=3, beta=(1,2,4): until eps~0.007). Rigorous: ridge Rayleigh bound O(eps) (via Thm E), lambda_max&gt;=(mu/eps-2mu)/|alpha|^2, K=1. Heuristic/numerical: middle tier, eigenvector convergence. See problem12_degenerate_directions.md REASSESSMENT 25 Oct: Herrera-Marin II (2609.38267) Sec 5 reports numerically an 'almost flat direction' from K~5 when fitting sums of exponentials to a long-memory kernel (slow poles trade mass with the baseline; not proved, misspecified setting). Same mechanism as my Problem 2 for the well-specified dictionary (lambda_min(I) falls ~10x per added exponential at r=2). Only a LOWER bound on lambda_min is proved here (Theorem T); a matching UPPER bound as K or the grid ratio grows would turn the flat direction into a theorem.</t>
+          <t>Draft done 2026-10-25 (needs your re-derivation). I(theta*) has three tiers: top ~1/eps along grad_alpha n=(1/beta_k) (pure n-direction, best determined); K-1 middle 'kernel-shape' directions (sum w_k/beta_k=0) of size O(1) set by the beta-grid via the Hawkes-corrected spectral Gram (checked: 0.0667 pred vs 0.0661 MC, K=2); ridge ~ eps/(mu(k-1)) along (1,-eps*alpha/mu) = mean-rate-preserving mu-n trade (E lam=mu/eps fixed, shape fixed). As eps-&gt;0 the RIDGE is the degenerate direction; at moderate eps for K&gt;=3 / tight grids a time-scale MIXTURE is smaller (K=3, beta=(1,2,4): until eps~0.007). Rigorous: ridge Rayleigh bound O(eps) (via Thm E), lambda_max&gt;=(mu/eps-2mu)/|alpha|^2, K=1. Heuristic/numerical: middle tier, eigenvector convergence. See problem12_degenerate_directions.md REASSESSMENT 25 Oct: Herrera-Marin II (2609.38267) Sec 5 reports numerically an 'almost flat direction' from K~5 when fitting sums of exponentials to a long-memory kernel (slow poles trade mass with the baseline; not proved, misspecified setting). Same mechanism as my Problem 2 for the well-specified dictionary (lambda_min(I) falls ~10x per added exponential at r=2). Only a LOWER bound on lambda_min is proved here (Theorem T); a matching UPPER bound as K or the grid ratio grows would turn the flat direction into a theorem. STRENGTHENED 25 Oct (tangent_bound.md): by Weyl, EVERY eigenvalue of I is bounded below rigorously (bound/MC = 0.23-0.85): top ~1/eps, middle O(1) independent of eps, ridge &gt;= ~0.25 eps. Upper bounds (ridge Rayleigh) and eigenvector convergence still numerical.</t>
         </is>
       </c>
     </row>
@@ -1499,10 +1499,14 @@
       </c>
       <c r="L14" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M14" s="33" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M14" s="33" t="inlineStr">
+        <is>
+          <t>First pass 2026-10-25. Theorem TR (expectation, realised-information norm, forgetting recursion F_i=(1-eta)F_{i-1}+dF_i, step-hold drift): avg E||v||^2_F &lt;= (2/(eta n))U_1 + (2/eta){C_q c+ kappa_x[d(-ln(1-eta))+Lambda_n/n] + C_d[(c_I/(eta c-))avg||d_i||^2_I + F_0 term]}; Corollary in I-norm with eta*F&gt;=c_F*I: eta*sigma^2 + (4 c_I/(c_F c-)) avg||d||^2/eta^2 (smooth: Delta^2/eta^2; jumps: J D^2/(eta^2 n), conservative vs sharp 1/eta). New ingredient: discounted log-det trace lemma. Every step checked numerically (K=1, alpha unknown): identity E&lt;g,v&gt;=E v'dF v, chain bound holds 9-21x slack, trace lemma holds. Assumptions A1-A4 (leverage, gap leverage xbar, info envelope, info lower bound c_F) MEASURED: inside window xbar&lt;=0.2, c_F&gt;=0.15; outside xbar max&gt;1, c_F min 0.05. Not done: derive A2/A4 (needs discount window &gt; mixing time ~ eps^2), sharp jump rate, K&gt;=2 numerics, constants 10-100x loose. See problem13_tracking_bound.md</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="33" customHeight="1" s="27">
       <c r="A15" s="29" t="n">
@@ -1618,7 +1622,7 @@
       </c>
       <c r="M16" s="33" t="inlineStr">
         <is>
-          <t>Draft done 2026-10-25, CONDITIONAL on Problem 13 (tracking bound not proved; built on measured MSE structure from P14). MSE(eta)=a*eta+B(eta), a=r/(2*eff). Smooth drift fast regime: eta*=(Delta_e^2/a)^(1/3) ~ eps^(4/3)*Delta^(2/3) (k&gt;1), MSE*=1.5*a*eta*; jumps: eta*=D*mu/sqrt(2*a*L_e) ~ eps^(3/2); k&lt;1 exponents 1+k/3, 1+k/2. Window cap eta&lt;=theta*mu^2/a ~ eps^2 binds as eps-&gt;0. Tracking beats static estimator only if P*eff*(A*mu)^2 &gt;~ 16 (checked: 8.7 no gain, 22.6 modest, 34.7 gain 26%). alpha unknown shifts eta* down by ~k^(-1/3). Sim (K=1): smooth alpha-known eta_opt 0.00292/0.00179/0.00089 vs predicted 0.00295/0.00193/0.00095 at eps 0.4/0.3/0.2; jumps within 15-27%. Not done: K&gt;=2 eta_opt, eps&lt;0.2, pure power-law regime. See problem15_step_size.md</t>
+          <t>Draft done 2026-10-25, CONDITIONAL on Problem 13 (tracking bound not proved; built on measured MSE structure from P14). MSE(eta)=a*eta+B(eta), a=r/(2*eff). Smooth drift fast regime: eta*=(Delta_e^2/a)^(1/3) ~ eps^(4/3)*Delta^(2/3) (k&gt;1), MSE*=1.5*a*eta*; jumps: eta*=D*mu/sqrt(2*a*L_e) ~ eps^(3/2); k&lt;1 exponents 1+k/3, 1+k/2. Window cap eta&lt;=theta*mu^2/a ~ eps^2 binds as eps-&gt;0. Tracking beats static estimator only if P*eff*(A*mu)^2 &gt;~ 16 (checked: 8.7 no gain, 22.6 modest, 34.7 gain 26%). alpha unknown shifts eta* down by ~k^(-1/3). Sim (K=1): smooth alpha-known eta_opt 0.00292/0.00179/0.00089 vs predicted 0.00295/0.00193/0.00095 at eps 0.4/0.3/0.2; jumps within 15-27%. Not done: K&gt;=2 eta_opt, eps&lt;0.2, pure power-law regime. See problem15_step_size.md UPDATE: Problem 13 first pass now exists (Theorem TR, constants 10-100x loose), so P15's formulas remain fitted to measured MSE; the P13 assumptions A2/A4 degrade exactly outside the window eta&lt;=theta*mu^2/a.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verification record (34 symbolic identities, 18 inequality families) and complexity improvements (O(K^4) moments, Newton multiplier search, Brent for the tangent bound)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -849,7 +849,7 @@
       </c>
       <c r="M3" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem02_identifiability.md; code/p2_window_bound.py, p2_lemma3_check.py, p2_gram_bound.py, p2_truncation_check.py, p2_truncation_bound.py. Fixed a thinning bug in p2_identifiability.py (had made lam_min ~10x too small for K&gt;=2). Findings (mu=1, beta=r^(k-1), MC 60-80k events): K&gt;=2 lam_min does NOT shrink with eps (K=2: ~0.045 at r=2, ~0.065 at r=4), cond ~ 1/eps (K=1: eps^-2); lam_min falls ~10x per added exponential (r=2: 0.069, 0.046, 0.0045 for K=1,2,3 at eps=0.1). Lower bounds: (1) Gram-matrix route is rigorous but useless (1e-6 to 1e-16 of truth, decays like eps^(2K+1)). (2) Theorem T (truncation + Lemma-B moments): lam_min(I) &gt;= (1/L)[lam_min(M) - sqrt(E|a|^4) sqrt(E lam^p / L^p)], M = E[a a^T] exact via a K^2 linear system (matches MC to 1-3%); bound is 2e-3 to 5e-2 of the MC lam_min for K&lt;=3 and non-vacuous; pure truncation without tail penalty would be within 2-8x. Open: closed-form formula in K and grid ratio, sharper tail bound, eps-sharpness for K&gt;=2. Depends on Lemma B (Problem 3 draft). Draft, not independently verified. CLOSED 25 Oct (Done): closed-form chain in K and grid ratio r: Cov(S) &gt;= (E lam/4) G (G=1/(b_i+b_j), spectral), exact E S_k = mu/(eps b_k), lam_min(M) &gt;= lam_min(C)/(1+2|m|^2), Cauchy inverse in closed form, then truncation with Lemma-1' moments; valid but 1e3-1e8 below truth (code/p2_closed_chain.py). Sharp scaling = three-tier structure (Problem 12), heuristic. STRENGTHENED 25 Oct (tangent_bound.md): tangent-line minorant I &gt;= (2/l0)M - (1/l0^2)M3 with exact moment systems (orders&lt;=3) gives a rigorous lower bound within 1.3-3.5x of Monte Carlo (K=1,2,3), correct eps-scaling (~0.25 eps); was 1e3-1e8 loose.</t>
+          <t>25 Oct 2026. problem02_identifiability.md; code/p2_window_bound.py, p2_lemma3_check.py, p2_gram_bound.py, p2_truncation_check.py, p2_truncation_bound.py. Fixed a thinning bug in p2_identifiability.py (had made lam_min ~10x too small for K&gt;=2). Findings (mu=1, beta=r^(k-1), MC 60-80k events): K&gt;=2 lam_min does NOT shrink with eps (K=2: ~0.045 at r=2, ~0.065 at r=4), cond ~ 1/eps (K=1: eps^-2); lam_min falls ~10x per added exponential (r=2: 0.069, 0.046, 0.0045 for K=1,2,3 at eps=0.1). Lower bounds: (1) Gram-matrix route is rigorous but useless (1e-6 to 1e-16 of truth, decays like eps^(2K+1)). (2) Theorem T (truncation + Lemma-B moments): lam_min(I) &gt;= (1/L)[lam_min(M) - sqrt(E|a|^4) sqrt(E lam^p / L^p)], M = E[a a^T] exact via a K^2 linear system (matches MC to 1-3%); bound is 2e-3 to 5e-2 of the MC lam_min for K&lt;=3 and non-vacuous; pure truncation without tail penalty would be within 2-8x. Open: closed-form formula in K and grid ratio, sharper tail bound, eps-sharpness for K&gt;=2. Depends on Lemma B (Problem 3 draft). Draft, not independently verified. CLOSED 25 Oct (Done): closed-form chain in K and grid ratio r: Cov(S) &gt;= (E lam/4) G (G=1/(b_i+b_j), spectral), exact E S_k = mu/(eps b_k), lam_min(M) &gt;= lam_min(C)/(1+2|m|^2), Cauchy inverse in closed form, then truncation with Lemma-1' moments; valid but 1e3-1e8 below truth (code/p2_closed_chain.py). Sharp scaling = three-tier structure (Problem 12), heuristic. STRENGTHENED 25 Oct (tangent_bound.md): tangent-line minorant I &gt;= (2/l0)M - (1/l0^2)M3 with exact moment systems (orders&lt;=3) gives a rigorous lower bound within 1.3-3.5x of Monte Carlo (K=1,2,3), correct eps-scaling (~0.25 eps); was 1e3-1e8 loose. COMPLEXITY 25 Oct: moments of order &lt;=3 by Kronecker-sum diagonalisation, O(K^4) time / O(K^3) memory (was O(K^9) / O(K^6)); lambda0-search by Brent (concavity in 1/lambda0), 13-26 evaluations (was 75).</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="M5" s="33" t="inlineStr">
         <is>
-          <t>24-25 Oct 2026. problem04_projection.md, code/p4_projection.py. Exact projection onto {mu&gt;=mu_min, alpha&gt;=0, sum alpha_k/beta_k&lt;=1-eps} in a DIAGONAL metric: mu separable; alpha_k = max(0, y_k - tau*w_k/d_k), tau from sorted breakpoints, O(K log K); matches SLSQP on 300 random instances (4e-6); &lt;1 ms for K up to 1e4. Regret-constant effect: non-expansive in the update's own metric, so no extra constant; the cost is cond(D^-1/2 I D^-1/2). K=1: universal ~5.83 (rho^2-&gt;1/2), independent of eps (raw ~1e6 at eps=1e-3). K&gt;=2 (corrected 25 Oct after fixing a simulator bug): scaled cond only 1.2-3x below raw and still grows as eps falls (K=2,r=2: 118-&gt;368; K=3: 765-&gt;2477), so a diagonal metric is NOT enough for K&gt;=2. Open: dense-metric projection (QP, ~O(K^2)), O(K) version, K&gt;=2 preconditioner. Status In progress because 'Done when' asks for the Fisher/ONS metric. UPDATE 25 Oct (problem05_circularity.md): for K=1 the diagonal clip is NOT adequate: it violates non-expansiveness in 0.7-4.6% of steps and inflates regret ~10x when the box is tight (E R_n 16 vs 3.5 at eps=.1; 79 vs 5.4 at eps=.03). Exact F-norm projection onto a box is O(1) for K=1 (edge minimisers + corners) and had 0 violations in 24 configs. Use it. CLOSED 25 Oct (Done): dense F-norm projection for any K (BVLS + bisection on the budget multiplier): matches brute force to 5e-14, non-expansive (0 violations in 2000 pairs), O(K^3) per inner solve (19 ms K=2, 97 ms K=5); the diagonal O(K log K) algorithm remains for the diagonal metric (code/p4_dense_projection.py).</t>
+          <t>24-25 Oct 2026. problem04_projection.md, code/p4_projection.py. Exact projection onto {mu&gt;=mu_min, alpha&gt;=0, sum alpha_k/beta_k&lt;=1-eps} in a DIAGONAL metric: mu separable; alpha_k = max(0, y_k - tau*w_k/d_k), tau from sorted breakpoints, O(K log K); matches SLSQP on 300 random instances (4e-6); &lt;1 ms for K up to 1e4. Regret-constant effect: non-expansive in the update's own metric, so no extra constant; the cost is cond(D^-1/2 I D^-1/2). K=1: universal ~5.83 (rho^2-&gt;1/2), independent of eps (raw ~1e6 at eps=1e-3). K&gt;=2 (corrected 25 Oct after fixing a simulator bug): scaled cond only 1.2-3x below raw and still grows as eps falls (K=2,r=2: 118-&gt;368; K=3: 765-&gt;2477), so a diagonal metric is NOT enough for K&gt;=2. Open: dense-metric projection (QP, ~O(K^2)), O(K) version, K&gt;=2 preconditioner. Status In progress because 'Done when' asks for the Fisher/ONS metric. UPDATE 25 Oct (problem05_circularity.md): for K=1 the diagonal clip is NOT adequate: it violates non-expansiveness in 0.7-4.6% of steps and inflates regret ~10x when the box is tight (E R_n 16 vs 3.5 at eps=.1; 79 vs 5.4 at eps=.03). Exact F-norm projection onto a box is O(1) for K=1 (edge minimisers + corners) and had 0 violations in 24 configs. Use it. CLOSED 25 Oct (Done): dense F-norm projection for any K (BVLS + bisection on the budget multiplier): matches brute force to 5e-14, non-expansive (0 violations in 2000 pairs), O(K^3) per inner solve (19 ms K=2, 97 ms K=5); the diagonal O(K log K) algorithm remains for the diagonal metric (code/p4_dense_projection.py). COMPLEXITY 25 Oct (verification_and_complexity.md): dense F-projection now uses safeguarded Newton on the budget multiplier (2-7 inner box-QP solves instead of 55-90; x15-30 faster, same solution to 1.7e-13). Estimator memory O(K^2), state O(K), per-event O(qK^2 + K^3).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Problems 12, 14, 11: three-tier theorem, tracking theorem with amplitude-effect closed forms, observed-information rate and non-consistency
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1382,7 +1382,7 @@
       </c>
       <c r="M12" s="33" t="inlineStr">
         <is>
-          <t>Draft done 2026-10-25 (needs your re-derivation). DECISION: C4 uses STATIONARY observation, dichotomy = bounded vs divergent. Rigorous: K=1 full dichotomy (Thm A, B); ANY K with k_K=2*mu*sum(alpha/beta^2)/n: E[1/lam]=O(eps) if k_K&gt;1 (Thm E, corrected Lyapunov log W+psi/W^2 with Perron weights) =&gt; no consistent mu-estimator (Cor E'); E[1/lam]&gt;=c eps^(k_K+eta) if k_K&lt;1 (Thm F) =&gt; alpha-known information diverges. Pathwise check of generator bounds passed. Open: efficient (alpha-unknown) info divergence for K&gt;=2 (numerics eff/m-&gt;1), matching upper bound/estimator (MLE is mixed-normal: observed info random, CV~0.5), k_K=1 borderline, cold-start coefficients. See problem11_dichotomy.md LITERATURE 25 Oct: divergence of mu-information for kappa&lt;=1 is Herrera-Marin Remark 4.8 (Fatou); he states the kappa&gt;1 direction is NOT proved. Gamma shape/Feller threshold k=2*beta*mu/alpha^2 confirmed against Jaisson-Rosenbaum Thm 2.2 (shape 2m*mu; tested, autocorrelation exp(-eps*beta*t) also confirmed). REASSESSMENT 25 Oct: divergence half = Herrera-Marin Remark 4.8; he leaves the converse (kappa&gt;1) unproved. Other session's Theorem A (K=1, stationary) claims it with rates (I have NOT verified its proof). Exact slopes of (1/2) log det I vs log(1/eps): 0.347,0.397,0.404,0.403,0.402 -&gt; (1-k0)/2=0.40 for k0=0.2; -&gt; 0 for k0&gt;=2. K=2 dictionary: A_T matches the K=1 value at equal k=2*mu*m (1.29/1.53/1.79 vs 1.26/1.55/1.78): supports threshold 2*mu*sum(w_k/beta_k)=1. Observation model matters (stationary vs empty start). VERIFICATION 25 Oct (verification_thmA_E_F.md): Lemma H re-derived and holds pathwise in 30/30 (parameter,z) cases; Theorems E and F re-derived: CORRECT given Lemma H; E_pi[A f]=0 and the E/F integral inequalities confirmed by stationary MC (16 independent replicates). GAP in the use of E: Corollary E'/Theorem B compare path laws with the SAME initial state; impossibility is rigorous for the experiment where S_0 (pre-sample history) is given, but for a stationary record with unobserved past one also needs KL(pi_theta||pi_theta') = O(1) (Gamma approx 0.003-0.034; not proved) - same step Herrera-Marin I calls open. Also: the empty-start experiment (the actual streaming setting) has mu-information &gt;= ln T for every k, so the 'mu unlearnable' headline is observation-model specific. UPDATE 25 Oct (theoremA_step2_and_stationary_tv.md): initial-state gap closed for K=1, k0&gt;1: TV(Q,Q') &lt;= sqrt(rho u'I_T u/2) + TV(pi,pi') (Lemma R), and TV(pi_theta,pi_theta') &lt;= C|delta| + C eps^min(1,k0-1/2) via exact characteristic function phi=G*Ftilde (Gamma comparator), imaginary-axis bound |D_eps(-i tau)|&lt;=31.5/alpha, monotone |phi|, and TV &lt;= ||.||_H1/(2 sqrt2). Numerics (FFT inversion of exact ch.f.): TV(pi,pi') = 0.026/0.070 for delta=0.1/0.3, flat in eps from 0.1 to 0.003; TV(pi,Gamma) ~ eps. MY PROOF, NOT REVIEWED; constants not explicit; K&gt;=2, k0&lt;=1 not covered. UPDATE 25 Oct (general_K_impossibility.md): impossibility of consistent mu-estimation for the STATIONARY record with unobserved past now proved for ANY K with k_K&gt;1 (Theorem V: TV(Q,Q') &lt;= C delta sqrt(ln(1/delta))), by a route that bypasses TV(pi_theta,pi_theta'): (1) KL of stationary theta-process vs theta'-dynamics started from pi_theta over a window L+T=O(1/gamma) is O(delta^2) via Theorem E; (2) superposition: process from state s = empty-start + ghost immigrants g_s(t); (3) cluster survival q(s)&lt;=C' gamma e^{-gamma s} from the flow Y'=-BY+alpha(1-e^{-|Y|}) and zeta'=-gamma zeta - r(|Y|) (first-moment bound would lose ln(1/eps)). Verified: flow vs cluster MC (K=1,2), ghost-hit prob decays e^{-gamma L} (K=2 sim). MY PROOF, UNREVIEWED. TV(pi,pi') for K&gt;=2 itself still open. LITERATURE 25 Oct (literature_search_report.md): CIR side: information about the drift constant finite iff a &gt; sigma (Ben Alaya et al. Thm 2.1); MLE defined only for 2a &gt; sigma^2 (Dehtiar et al.); critical case sqrt(log T) rate. Discrete side: all estimation results found are CLSE/OLS; Li 2011: nonzero initial values =&gt; CLSE of immigration mean inconsistent; Anne-Lu-Yu-Zhou 2026: OLS intercept inconsistent in local-to-unity affine processes (no Hawkes, no information bound; overlap risk Medium). Herrera-Marin's Wei-Winnicki attribution UNVERIFIED. THM T CONSTANTS 25 Oct (thmT_explicit_constants.md): Theorem T now has an explicit chain: |d|&lt;=19 (true sup 1.143), tail exponent q=k0/(2(1+3/X0))&gt;1/2 (k/(1+r)^2=k0 exactly), certified TV(pi,Gamma)&lt;=Phi/(2 sqrt2); k0=2: 2e-2 (eps=1e-4), 1e-3 (1e-5), 8.6e-5 (1e-6); bound 1e2-1e3 above truth, valid in all tests. Ridge pair: TV&lt;=2.4e-3+0.39 delta (eps&lt;=1e-5, k0=2, delta&lt;=0.3). Phi by floating-point quadrature of hand-proved majorants, not interval arithmetic; KL step evaluated on a grid; informative only for eps&lt;~1e-4. FINAL AUDIT 25 Oct (final_audit.md): the 'no consistent estimator given S0' statements (Thm B, Cor D, Cor E') were stronger than the KL lemma proves: the correct bound is TV(Q) &lt;= TV(pi_theta, pi_theta') + sqrt(rho T u'Iu/2). Rigorous impossibility: K=1 stationary record (Thm T), any K stationary record with unobserved past (Thm V). K&gt;=2 with S0 observed: open.</t>
+          <t>Draft done 2026-10-25 (needs your re-derivation). DECISION: C4 uses STATIONARY observation, dichotomy = bounded vs divergent. Rigorous: K=1 full dichotomy (Thm A, B); ANY K with k_K=2*mu*sum(alpha/beta^2)/n: E[1/lam]=O(eps) if k_K&gt;1 (Thm E, corrected Lyapunov log W+psi/W^2 with Perron weights) =&gt; no consistent mu-estimator (Cor E'); E[1/lam]&gt;=c eps^(k_K+eta) if k_K&lt;1 (Thm F) =&gt; alpha-known information diverges. Pathwise check of generator bounds passed. Open: efficient (alpha-unknown) info divergence for K&gt;=2 (numerics eff/m-&gt;1), matching upper bound/estimator (MLE is mixed-normal: observed info random, CV~0.5), k_K=1 borderline, cold-start coefficients. See problem11_dichotomy.md LITERATURE 25 Oct: divergence of mu-information for kappa&lt;=1 is Herrera-Marin Remark 4.8 (Fatou); he states the kappa&gt;1 direction is NOT proved. Gamma shape/Feller threshold k=2*beta*mu/alpha^2 confirmed against Jaisson-Rosenbaum Thm 2.2 (shape 2m*mu; tested, autocorrelation exp(-eps*beta*t) also confirmed). REASSESSMENT 25 Oct: divergence half = Herrera-Marin Remark 4.8; he leaves the converse (kappa&gt;1) unproved. Other session's Theorem A (K=1, stationary) claims it with rates (I have NOT verified its proof). Exact slopes of (1/2) log det I vs log(1/eps): 0.347,0.397,0.404,0.403,0.402 -&gt; (1-k0)/2=0.40 for k0=0.2; -&gt; 0 for k0&gt;=2. K=2 dictionary: A_T matches the K=1 value at equal k=2*mu*m (1.29/1.53/1.79 vs 1.26/1.55/1.78): supports threshold 2*mu*sum(w_k/beta_k)=1. Observation model matters (stationary vs empty start). VERIFICATION 25 Oct (verification_thmA_E_F.md): Lemma H re-derived and holds pathwise in 30/30 (parameter,z) cases; Theorems E and F re-derived: CORRECT given Lemma H; E_pi[A f]=0 and the E/F integral inequalities confirmed by stationary MC (16 independent replicates). GAP in the use of E: Corollary E'/Theorem B compare path laws with the SAME initial state; impossibility is rigorous for the experiment where S_0 (pre-sample history) is given, but for a stationary record with unobserved past one also needs KL(pi_theta||pi_theta') = O(1) (Gamma approx 0.003-0.034; not proved) - same step Herrera-Marin I calls open. Also: the empty-start experiment (the actual streaming setting) has mu-information &gt;= ln T for every k, so the 'mu unlearnable' headline is observation-model specific. UPDATE 25 Oct (theoremA_step2_and_stationary_tv.md): initial-state gap closed for K=1, k0&gt;1: TV(Q,Q') &lt;= sqrt(rho u'I_T u/2) + TV(pi,pi') (Lemma R), and TV(pi_theta,pi_theta') &lt;= C|delta| + C eps^min(1,k0-1/2) via exact characteristic function phi=G*Ftilde (Gamma comparator), imaginary-axis bound |D_eps(-i tau)|&lt;=31.5/alpha, monotone |phi|, and TV &lt;= ||.||_H1/(2 sqrt2). Numerics (FFT inversion of exact ch.f.): TV(pi,pi') = 0.026/0.070 for delta=0.1/0.3, flat in eps from 0.1 to 0.003; TV(pi,Gamma) ~ eps. MY PROOF, NOT REVIEWED; constants not explicit; K&gt;=2, k0&lt;=1 not covered. UPDATE 25 Oct (general_K_impossibility.md): impossibility of consistent mu-estimation for the STATIONARY record with unobserved past now proved for ANY K with k_K&gt;1 (Theorem V: TV(Q,Q') &lt;= C delta sqrt(ln(1/delta))), by a route that bypasses TV(pi_theta,pi_theta'): (1) KL of stationary theta-process vs theta'-dynamics started from pi_theta over a window L+T=O(1/gamma) is O(delta^2) via Theorem E; (2) superposition: process from state s = empty-start + ghost immigrants g_s(t); (3) cluster survival q(s)&lt;=C' gamma e^{-gamma s} from the flow Y'=-BY+alpha(1-e^{-|Y|}) and zeta'=-gamma zeta - r(|Y|) (first-moment bound would lose ln(1/eps)). Verified: flow vs cluster MC (K=1,2), ghost-hit prob decays e^{-gamma L} (K=2 sim). MY PROOF, UNREVIEWED. TV(pi,pi') for K&gt;=2 itself still open. LITERATURE 25 Oct (literature_search_report.md): CIR side: information about the drift constant finite iff a &gt; sigma (Ben Alaya et al. Thm 2.1); MLE defined only for 2a &gt; sigma^2 (Dehtiar et al.); critical case sqrt(log T) rate. Discrete side: all estimation results found are CLSE/OLS; Li 2011: nonzero initial values =&gt; CLSE of immigration mean inconsistent; Anne-Lu-Yu-Zhou 2026: OLS intercept inconsistent in local-to-unity affine processes (no Hawkes, no information bound; overlap risk Medium). Herrera-Marin's Wei-Winnicki attribution UNVERIFIED. THM T CONSTANTS 25 Oct (thmT_explicit_constants.md): Theorem T now has an explicit chain: |d|&lt;=19 (true sup 1.143), tail exponent q=k0/(2(1+3/X0))&gt;1/2 (k/(1+r)^2=k0 exactly), certified TV(pi,Gamma)&lt;=Phi/(2 sqrt2); k0=2: 2e-2 (eps=1e-4), 1e-3 (1e-5), 8.6e-5 (1e-6); bound 1e2-1e3 above truth, valid in all tests. Ridge pair: TV&lt;=2.4e-3+0.39 delta (eps&lt;=1e-5, k0=2, delta&lt;=0.3). Phi by floating-point quadrature of hand-proved majorants, not interval arithmetic; KL step evaluated on a grid; informative only for eps&lt;~1e-4. FINAL AUDIT 25 Oct (final_audit.md): the 'no consistent estimator given S0' statements (Thm B, Cor D, Cor E') were stronger than the KL lemma proves: the correct bound is TV(Q) &lt;= TV(pi_theta, pi_theta') + sqrt(rho T u'Iu/2). Rigorous impossibility: K=1 stationary record (Thm T), any K stationary record with unobserved past (Thm V). K&gt;=2 with S0 observed: open. MATCHING RATE / NON-CONSISTENCY 25 Oct (problem11_observed_information.md): Theorem UB: |mu_hat - mu| &lt;= C sqrt(loglog I_T)/sqrt(I_T) on {I_T &gt;= M0} (observed information, any k); Theorem NC: at eps=c/T NO estimator is consistent for ANY k (stopped-KL bounded pathwise on an event of probability &gt;= p &gt; 0), so divergence of expected information for k&lt;1 does not give consistency; simulations: P(|err|&gt;mu/2) = 0.40 (k=0.6), 0.34 (k=2), flat in T.</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="M13" s="33" t="inlineStr">
         <is>
-          <t>Draft done 2026-10-25 (needs your re-derivation). I(theta*) has three tiers: top ~1/eps along grad_alpha n=(1/beta_k) (pure n-direction, best determined); K-1 middle 'kernel-shape' directions (sum w_k/beta_k=0) of size O(1) set by the beta-grid via the Hawkes-corrected spectral Gram (checked: 0.0667 pred vs 0.0661 MC, K=2); ridge ~ eps/(mu(k-1)) along (1,-eps*alpha/mu) = mean-rate-preserving mu-n trade (E lam=mu/eps fixed, shape fixed). As eps-&gt;0 the RIDGE is the degenerate direction; at moderate eps for K&gt;=3 / tight grids a time-scale MIXTURE is smaller (K=3, beta=(1,2,4): until eps~0.007). Rigorous: ridge Rayleigh bound O(eps) (via Thm E), lambda_max&gt;=(mu/eps-2mu)/|alpha|^2, K=1. Heuristic/numerical: middle tier, eigenvector convergence. See problem12_degenerate_directions.md REASSESSMENT 25 Oct: Herrera-Marin II (2609.38267) Sec 5 reports numerically an 'almost flat direction' from K~5 when fitting sums of exponentials to a long-memory kernel (slow poles trade mass with the baseline; not proved, misspecified setting). Same mechanism as my Problem 2 for the well-specified dictionary (lambda_min(I) falls ~10x per added exponential at r=2). Only a LOWER bound on lambda_min is proved here (Theorem T); a matching UPPER bound as K or the grid ratio grows would turn the flat direction into a theorem. STRENGTHENED 25 Oct (tangent_bound.md): by Weyl, EVERY eigenvalue of I is bounded below rigorously (bound/MC = 0.23-0.85): top ~1/eps, middle O(1) independent of eps, ridge &gt;= ~0.25 eps. Upper bounds (ridge Rayleigh) and eigenvector convergence still numerical.</t>
+          <t>Draft done 2026-10-25 (needs your re-derivation). I(theta*) has three tiers: top ~1/eps along grad_alpha n=(1/beta_k) (pure n-direction, best determined); K-1 middle 'kernel-shape' directions (sum w_k/beta_k=0) of size O(1) set by the beta-grid via the Hawkes-corrected spectral Gram (checked: 0.0667 pred vs 0.0661 MC, K=2); ridge ~ eps/(mu(k-1)) along (1,-eps*alpha/mu) = mean-rate-preserving mu-n trade (E lam=mu/eps fixed, shape fixed). As eps-&gt;0 the RIDGE is the degenerate direction; at moderate eps for K&gt;=3 / tight grids a time-scale MIXTURE is smaller (K=3, beta=(1,2,4): until eps~0.007). Rigorous: ridge Rayleigh bound O(eps) (via Thm E), lambda_max&gt;=(mu/eps-2mu)/|alpha|^2, K=1. Heuristic/numerical: middle tier, eigenvector convergence. See problem12_degenerate_directions.md REASSESSMENT 25 Oct: Herrera-Marin II (2609.38267) Sec 5 reports numerically an 'almost flat direction' from K~5 when fitting sums of exponentials to a long-memory kernel (slow poles trade mass with the baseline; not proved, misspecified setting). Same mechanism as my Problem 2 for the well-specified dictionary (lambda_min(I) falls ~10x per added exponential at r=2). Only a LOWER bound on lambda_min is proved here (Theorem T); a matching UPPER bound as K or the grid ratio grows would turn the flat direction into a theorem. STRENGTHENED 25 Oct (tangent_bound.md): by Weyl, EVERY eigenvalue of I is bounded below rigorously (bound/MC = 0.23-0.85): top ~1/eps, middle O(1) independent of eps, ridge &gt;= ~0.25 eps. Upper bounds (ridge Rayleigh) and eigenvector convergence still numerical. THREE-TIER THEOREM 25 Oct (problem12_upper_bounds.md): fast modes y_j = sum alpha_k S_k/(beta_k - a_j) satisfy A y_j = -a_j y_j + mu exactly; Lyapunov y_j^2/W gives E[y_j^2/lam] = O(1) uniformly in eps =&gt; middle eigenvalues bounded above and below (both eps-independent), top Theta(1/eps), ridge O(eps); smallest eigenvector -&gt; ridge direction at rate O(eps/g) (Davis-Kahan); symbolic + pathwise checks pass; constants ~20x loose.</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="M14" s="33" t="inlineStr">
         <is>
-          <t>First pass 2026-10-25. Theorem TR (expectation, realised-information norm, forgetting recursion F_i=(1-eta)F_{i-1}+dF_i, step-hold drift): avg E||v||^2_F &lt;= (2/(eta n))U_1 + (2/eta){C_q c+ kappa_x[d(-ln(1-eta))+Lambda_n/n] + C_d[(c_I/(eta c-))avg||d_i||^2_I + F_0 term]}; Corollary in I-norm with eta*F&gt;=c_F*I: eta*sigma^2 + (4 c_I/(c_F c-)) avg||d||^2/eta^2 (smooth: Delta^2/eta^2; jumps: J D^2/(eta^2 n), conservative vs sharp 1/eta). New ingredient: discounted log-det trace lemma. Every step checked numerically (K=1, alpha unknown): identity E&lt;g,v&gt;=E v'dF v, chain bound holds 9-21x slack, trace lemma holds. Assumptions A1-A4 (leverage, gap leverage xbar, info envelope, info lower bound c_F) MEASURED: inside window xbar&lt;=0.2, c_F&gt;=0.15; outside xbar max&gt;1, c_F min 0.05. Not done: derive A2/A4 (needs discount window &gt; mixing time ~ eps^2), sharp jump rate, K&gt;=2 numerics, constants 10-100x loose. See problem13_tracking_bound.md</t>
+          <t>SECOND PASS 2026-10-25 (problem13_second_pass.md): Theorem TR2 via exact recursion v_{i+1}=(I-G_i)(v_i-d_i)-F_i^-1 s_i (continuous drift, no step-hold), split v=v^xi+v^d + Minkowski: SHARP jump rate D^2/eta (measured slope -0.94), noise constant ~2x better; A1/A2 derived from A4 with explicit eta/eps^2 dependence (K=1); A4 proved for K=1 (stationary params) by window argument, window condition eta&lt;~eps^2/(kappa*mu*C). Checks K=1,2 (contraction lemma, exact split, leverage formulas, c_win scaling in T0*eps). STILL OPEN: A4 for K&gt;=2, smooth-drift constant ~25x loose, a.s. vs high-prob, diagonal clip not covered. First pass 2026-10-25. Theorem TR (expectation, realised-information norm, forgetting recursion F_i=(1-eta)F_{i-1}+dF_i, step-hold drift): avg E||v||^2_F &lt;= (2/(eta n))U_1 + (2/eta){C_q c+ kappa_x[d(-ln(1-eta))+Lambda_n/n] + C_d[(c_I/(eta c-))avg||d_i||^2_I + F_0 term]}; Corollary in I-norm with eta*F&gt;=c_F*I: eta*sigma^2 + (4 c_I/(c_F c-)) avg||d||^2/eta^2 (smooth: Delta^2/eta^2; jumps: J D^2/(eta^2 n), conservative vs sharp 1/eta). New ingredient: discounted log-det trace lemma. Every step checked numerically (K=1, alpha unknown): identity E&lt;g,v&gt;=E v'dF v, chain bound holds 9-21x slack, trace lemma holds. Assumptions A1-A4 (leverage, gap leverage xbar, info envelope, info lower bound c_F) MEASURED: inside window xbar&lt;=0.2, c_F&gt;=0.15; outside xbar max&gt;1, c_F min 0.05. Not done: derive A2/A4 (needs discount window &gt; mixing time ~ eps^2), sharp jump rate, K&gt;=2 numerics, constants 10-100x loose. See problem13_tracking_bound.md</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="M15" s="33" t="inlineStr">
         <is>
-          <t>DECISION 2026-10-25: bounded variation as piecewise-Lipschitz class (Lipschitz rate Delta, &lt;=J jumps of size &lt;=D, box mu_t in [mu,c_mu*mu], eps_t in [eps,c_eps*eps], fixed reference Fisher norm). Target for P13: eta*sigma^2 + Delta^2/eta^2 (response of a time-varying-gain filter, gain eta*mu_t/eps) + J*D^2/(eta*T); sigma^2=r/(2*eff) (K=1 alpha known: mu/(2*eps*m)). Verified numerically (causal sampling): sinusoid, triangle, ramp, random walk, jumps; K=1,2,3 (grids (1,2),(1,4),(1,2,4),(1,3,9)); noise coeff r/(2 eff) within 3-13% in window; linear window eta&lt;=theta_k*mu^2/a, theta_k~0.013-0.03 (k-dependent). Problem 5 recursion verbatim cannot track drift (needs forgetting). RETRACTED c_lag~1.8: extra lag for alpha-unknown is an amplitude effect of the data-driven preconditioner (1.3-1.75x at A=0.2-0.5, -&gt;1 as A-&gt;0), absent with fixed preconditioner. Metric equivalence kappa_I: K=1 7-9, K=2 10-11 (mu x1.5), eps-independent. Hall-Willett VERIFIED from LaTeX source (adversarial regret C(1+sum||lam_{t+1}-Phi_t(lam_t)||_2)*sqrt(T): variation measure is a path length relative to known dynamics, norm not squared; no parameter-drift model). Solo (Piggott-Solo ICASSP 2018) NOT read: closed access, no OA copy (needs your library). Open: K&gt;=4, eps&lt;0.4 for K&gt;=2, analytic derivation of the adaptive-preconditioner excess. See problem14_drift_model.md CLEANUP 25 Oct: stale c_lag / amplitude-independence / K=2 bias-ratio statements struck in the note; noise convention (sigma^2=a=r/(2 eff)); path-length bound V^2/(eta T) (factor 1/2 not derived); jump term units. Label clashes resolved in LABELS.md.</t>
+          <t>DECISION 2026-10-25: bounded variation as piecewise-Lipschitz class (Lipschitz rate Delta, &lt;=J jumps of size &lt;=D, box mu_t in [mu,c_mu*mu], eps_t in [eps,c_eps*eps], fixed reference Fisher norm). Target for P13: eta*sigma^2 + Delta^2/eta^2 (response of a time-varying-gain filter, gain eta*mu_t/eps) + J*D^2/(eta*T); sigma^2=r/(2*eff) (K=1 alpha known: mu/(2*eps*m)). Verified numerically (causal sampling): sinusoid, triangle, ramp, random walk, jumps; K=1,2,3 (grids (1,2),(1,4),(1,2,4),(1,3,9)); noise coeff r/(2 eff) within 3-13% in window; linear window eta&lt;=theta_k*mu^2/a, theta_k~0.013-0.03 (k-dependent). Problem 5 recursion verbatim cannot track drift (needs forgetting). RETRACTED c_lag~1.8: extra lag for alpha-unknown is an amplitude effect of the data-driven preconditioner (1.3-1.75x at A=0.2-0.5, -&gt;1 as A-&gt;0), absent with fixed preconditioner. Metric equivalence kappa_I: K=1 7-9, K=2 10-11 (mu x1.5), eps-independent. Hall-Willett VERIFIED from LaTeX source (adversarial regret C(1+sum||lam_{t+1}-Phi_t(lam_t)||_2)*sqrt(T): variation measure is a path length relative to known dynamics, norm not squared; no parameter-drift model). Solo (Piggott-Solo ICASSP 2018) NOT read: closed access, no OA copy (needs your library). Open: K&gt;=4, eps&lt;0.4 for K&gt;=2, analytic derivation of the adaptive-preconditioner excess. See problem14_drift_model.md CLEANUP 25 Oct: stale c_lag / amplitude-independence / K=2 bias-ratio statements struck in the note; noise convention (sigma^2=a=r/(2 eff)); path-length bound V^2/(eta T) (factor 1/2 not derived); jump term units. Label clashes resolved in LABELS.md. TRACKING THEOREM 25 Oct (problem14_tracking_theorem.md): pathwise recursion D_i &lt;= (1+rho)[(1-eta)D_{i-1} + X - 2&lt;g,v&gt; + G] + (1+1/rho)||d||^2_F, E[X - 2&lt;g,v&gt;] &lt;= E Xi; steady state E||v||^2_I &lt;~ 2 eta d + 4(||d||_I/eta)^2 (modulo window hypothesis W); checked in 57,616 gaps (0 violations; measured 0.0077 vs bound 0.0463). AMPLITUDE EFFECT derived: O(A^2) gain-modulation with closed forms C2_fixed, C2_adaptive (sympy), verified vs exact ODE to 4 digits; alpha-unknown matrix case: deterministic skeleton reproduces adaptive/fixed 1.11, 1.33, 1.67 (MC 1.32, 1.48, 1.75).</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="M16" s="33" t="inlineStr">
         <is>
-          <t>Draft done 2026-10-25, CONDITIONAL on Problem 13 (tracking bound not proved; built on measured MSE structure from P14). MSE(eta)=a*eta+B(eta), a=r/(2*eff). Smooth drift fast regime: eta*=(Delta_e^2/a)^(1/3) ~ eps^(4/3)*Delta^(2/3) (k&gt;1), MSE*=1.5*a*eta*; jumps: eta*=D*mu/sqrt(2*a*L_e) ~ eps^(3/2); k&lt;1 exponents 1+k/3, 1+k/2. Window cap eta&lt;=theta*mu^2/a ~ eps^2 binds as eps-&gt;0. Tracking beats static estimator only if P*eff*(A*mu)^2 &gt;~ 16 (checked: 8.7 no gain, 22.6 modest, 34.7 gain 26%). alpha unknown shifts eta* down by ~k^(-1/3). Sim (K=1): smooth alpha-known eta_opt 0.00292/0.00179/0.00089 vs predicted 0.00295/0.00193/0.00095 at eps 0.4/0.3/0.2; jumps within 15-27%. Not done: K&gt;=2 eta_opt, eps&lt;0.2, pure power-law regime. See problem15_step_size.md UPDATE: Problem 13 first pass now exists (Theorem TR, constants 10-100x loose), so P15's formulas remain fitted to measured MSE; the P13 assumptions A2/A4 degrade exactly outside the window eta&lt;=theta*mu^2/a.</t>
+          <t>Draft done 2026-10-25, CONDITIONAL on Problem 13 (tracking bound not proved; built on measured MSE structure from P14). MSE(eta)=a*eta+B(eta), a=r/(2*eff). Smooth drift fast regime: eta*=(Delta_e^2/a)^(1/3) ~ eps^(4/3)*Delta^(2/3) (k&gt;1), MSE*=1.5*a*eta*; jumps: eta*=D*mu/sqrt(2*a*L_e) ~ eps^(3/2); k&lt;1 exponents 1+k/3, 1+k/2. Window cap eta&lt;=theta*mu^2/a ~ eps^2 binds as eps-&gt;0. Tracking beats static estimator only if P*eff*(A*mu)^2 &gt;~ 16 (checked: 8.7 no gain, 22.6 modest, 34.7 gain 26%). alpha unknown shifts eta* down by ~k^(-1/3). Sim (K=1): smooth alpha-known eta_opt 0.00292/0.00179/0.00089 vs predicted 0.00295/0.00193/0.00095 at eps 0.4/0.3/0.2; jumps within 15-27%. Not done: K&gt;=2 eta_opt, eps&lt;0.2, pure power-law regime. See problem15_step_size.md UPDATE: Problem 13 first pass now exists (Theorem TR, constants 10-100x loose), so P15's formulas remain fitted to measured MSE; the P13 assumptions A2/A4 degrade exactly outside the window eta&lt;=theta*mu^2/a. UPDATE 2: P13 second pass proves the jump cost scales as D^2/eta (as assumed in P15's jump law) and shows the leverage assumptions hold iff eta&lt;~eps^2 (K=1), matching P15's window cap.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Problem 13 third pass: projection, high-probability, Step-3 constant, K>=2 A4, mu-drift; notes, code, tracker and LaTeX update
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1504,7 +1504,7 @@
       </c>
       <c r="M14" s="33" t="inlineStr">
         <is>
-          <t>SECOND PASS 2026-10-25 (problem13_second_pass.md): Theorem TR2 via exact recursion v_{i+1}=(I-G_i)(v_i-d_i)-F_i^-1 s_i (continuous drift, no step-hold), split v=v^xi+v^d + Minkowski: SHARP jump rate D^2/eta (measured slope -0.94), noise constant ~2x better; A1/A2 derived from A4 with explicit eta/eps^2 dependence (K=1); A4 proved for K=1 (stationary params) by window argument, window condition eta&lt;~eps^2/(kappa*mu*C). Checks K=1,2 (contraction lemma, exact split, leverage formulas, c_win scaling in T0*eps). STILL OPEN: A4 for K&gt;=2, smooth-drift constant ~25x loose, a.s. vs high-prob, diagonal clip not covered. First pass 2026-10-25. Theorem TR (expectation, realised-information norm, forgetting recursion F_i=(1-eta)F_{i-1}+dF_i, step-hold drift): avg E||v||^2_F &lt;= (2/(eta n))U_1 + (2/eta){C_q c+ kappa_x[d(-ln(1-eta))+Lambda_n/n] + C_d[(c_I/(eta c-))avg||d_i||^2_I + F_0 term]}; Corollary in I-norm with eta*F&gt;=c_F*I: eta*sigma^2 + (4 c_I/(c_F c-)) avg||d||^2/eta^2 (smooth: Delta^2/eta^2; jumps: J D^2/(eta^2 n), conservative vs sharp 1/eta). New ingredient: discounted log-det trace lemma. Every step checked numerically (K=1, alpha unknown): identity E&lt;g,v&gt;=E v'dF v, chain bound holds 9-21x slack, trace lemma holds. Assumptions A1-A4 (leverage, gap leverage xbar, info envelope, info lower bound c_F) MEASURED: inside window xbar&lt;=0.2, c_F&gt;=0.15; outside xbar max&gt;1, c_F min 0.05. Not done: derive A2/A4 (needs discount window &gt; mixing time ~ eps^2), sharp jump rate, K&gt;=2 numerics, constants 10-100x loose. See problem13_tracking_bound.md</t>
+          <t>SECOND PASS 2026-10-25 (problem13_second_pass.md): Theorem TR2 via exact recursion v_{i+1}=(I-G_i)(v_i-d_i)-F_i^-1 s_i (continuous drift, no step-hold), split v=v^xi+v^d + Minkowski: SHARP jump rate D^2/eta (measured slope -0.94), noise constant ~2x better; A1/A2 derived from A4 with explicit eta/eps^2 dependence (K=1); A4 proved for K=1 (stationary params) by window argument, window condition eta&lt;~eps^2/(kappa*mu*C). Checks K=1,2 (contraction lemma, exact split, leverage formulas, c_win scaling in T0*eps). STILL OPEN: A4 for K&gt;=2, smooth-drift constant ~25x loose, a.s. vs high-prob, diagonal clip not covered. First pass 2026-10-25. Theorem TR (expectation, realised-information norm, forgetting recursion F_i=(1-eta)F_{i-1}+dF_i, step-hold drift): avg E||v||^2_F &lt;= (2/(eta n))U_1 + (2/eta){C_q c+ kappa_x[d(-ln(1-eta))+Lambda_n/n] + C_d[(c_I/(eta c-))avg||d_i||^2_I + F_0 term]}; Corollary in I-norm with eta*F&gt;=c_F*I: eta*sigma^2 + (4 c_I/(c_F c-)) avg||d||^2/eta^2 (smooth: Delta^2/eta^2; jumps: J D^2/(eta^2 n), conservative vs sharp 1/eta). New ingredient: discounted log-det trace lemma. Every step checked numerically (K=1, alpha unknown): identity E&lt;g,v&gt;=E v'dF v, chain bound holds 9-21x slack, trace lemma holds. Assumptions A1-A4 (leverage, gap leverage xbar, info envelope, info lower bound c_F) MEASURED: inside window xbar&lt;=0.2, c_F&gt;=0.15; outside xbar max&gt;1, c_F min 0.05. Not done: derive A2/A4 (needs discount window &gt; mixing time ~ eps^2), sharp jump rate, K&gt;=2 numerics, constants 10-100x loose. See problem13_tracking_bound.md THIRD PASS 2026-10-25 (problem13_third_pass.md): projection proved for exact F-norm projection (diagonal clip NOT covered); high-prob A1' via predictable leverage/stopping (A2 overshoot step open); Step-3 constant derived line by line (valid, ~1e10 conservative); A4 for K&gt;=2 CONDITIONAL on U2 (kurtosis-type) and H1 (basis conditioning), K=2 numerics support; drift covered for mu-drift only (alpha fixed, box constant), alpha-drift open; projected jump-rate slope numerically noisy.</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="M16" s="33" t="inlineStr">
         <is>
-          <t>Draft done 2026-10-25, CONDITIONAL on Problem 13 (tracking bound not proved; built on measured MSE structure from P14). MSE(eta)=a*eta+B(eta), a=r/(2*eff). Smooth drift fast regime: eta*=(Delta_e^2/a)^(1/3) ~ eps^(4/3)*Delta^(2/3) (k&gt;1), MSE*=1.5*a*eta*; jumps: eta*=D*mu/sqrt(2*a*L_e) ~ eps^(3/2); k&lt;1 exponents 1+k/3, 1+k/2. Window cap eta&lt;=theta*mu^2/a ~ eps^2 binds as eps-&gt;0. Tracking beats static estimator only if P*eff*(A*mu)^2 &gt;~ 16 (checked: 8.7 no gain, 22.6 modest, 34.7 gain 26%). alpha unknown shifts eta* down by ~k^(-1/3). Sim (K=1): smooth alpha-known eta_opt 0.00292/0.00179/0.00089 vs predicted 0.00295/0.00193/0.00095 at eps 0.4/0.3/0.2; jumps within 15-27%. Not done: K&gt;=2 eta_opt, eps&lt;0.2, pure power-law regime. See problem15_step_size.md UPDATE: Problem 13 first pass now exists (Theorem TR, constants 10-100x loose), so P15's formulas remain fitted to measured MSE; the P13 assumptions A2/A4 degrade exactly outside the window eta&lt;=theta*mu^2/a. UPDATE 2: P13 second pass proves the jump cost scales as D^2/eta (as assumed in P15's jump law) and shows the leverage assumptions hold iff eta&lt;~eps^2 (K=1), matching P15's window cap.</t>
+          <t>Draft done 2026-10-25, CONDITIONAL on Problem 13 (tracking bound not proved; built on measured MSE structure from P14). MSE(eta)=a*eta+B(eta), a=r/(2*eff). Smooth drift fast regime: eta*=(Delta_e^2/a)^(1/3) ~ eps^(4/3)*Delta^(2/3) (k&gt;1), MSE*=1.5*a*eta*; jumps: eta*=D*mu/sqrt(2*a*L_e) ~ eps^(3/2); k&lt;1 exponents 1+k/3, 1+k/2. Window cap eta&lt;=theta*mu^2/a ~ eps^2 binds as eps-&gt;0. Tracking beats static estimator only if P*eff*(A*mu)^2 &gt;~ 16 (checked: 8.7 no gain, 22.6 modest, 34.7 gain 26%). alpha unknown shifts eta* down by ~k^(-1/3). Sim (K=1): smooth alpha-known eta_opt 0.00292/0.00179/0.00089 vs predicted 0.00295/0.00193/0.00095 at eps 0.4/0.3/0.2; jumps within 15-27%. Not done: K&gt;=2 eta_opt, eps&lt;0.2, pure power-law regime. See problem15_step_size.md UPDATE: Problem 13 first pass now exists (Theorem TR, constants 10-100x loose), so P15's formulas remain fitted to measured MSE; the P13 assumptions A2/A4 degrade exactly outside the window eta&lt;=theta*mu^2/a. UPDATE 2: P13 second pass proves the jump cost scales as D^2/eta (as assumed in P15's jump law) and shows the leverage assumptions hold iff eta&lt;~eps^2 (K=1), matching P15's window cap. Third pass of P13 (problem13_third_pass.md) does not change these formulas; they inherit its limits (exact projection only, mu-drift only, K&gt;=2 A4 conditional).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: mark Problems 6, 8, 9, 19, 22 In progress with what exists and what is missing
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1084,10 +1084,14 @@
       </c>
       <c r="L7" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M7" s="33" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="M7" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026. PARTIAL (problem05_E5_expected_regret.md, theoremR_proof_complete.md, K2_regret_chain.md, box_cost_and_lower_bound.md): Theorem R gives E R_T &lt;= (1/2 + O(delta+eta)) d ln T + C with C = O(mu d ln(1/(eps delta)) / (beta eps^2 delta^2)) (order only, K=1; general K with the tangent information level lambda_*/2); burn-in is ~1/eps^2 events (~1/(beta eps) in time units), not 1/(mu eps); no C log(1/eps) term visible in time units (leading term d/2 ln T + 1/2 ln det I with det I bounded for k0&gt;1). MISSING for Done: every constant of the theorem written as an explicit function of (eps, mu, K, beta-grid); the eps-dependence of C is an order, not a proved sharp rate.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="46.5" customHeight="1" s="27">
       <c r="A8" s="29" t="n">
@@ -1202,10 +1206,14 @@
       </c>
       <c r="L9" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M9" s="33" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="M9" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026. PARTIAL: the notion used throughout is the log-loss (KL) regret of a predictive intensity, E R_n = KL(P_theta^(n) || Q^(n)) (box_cost_and_lower_bound.md B1), with pseudo-regret R_n = sum int lam* psi(lam_theta/lam*) &lt;= X_n pathwise; parameter error enters via the Fisher-norm quantities D_n = ||theta_{n+1}-theta*||^2_{F_n} (Lemma C1) and the tracking theorem (problem14_tracking_theorem.md); the lower bound passes from KL to MSE through mutual information (Prop LB). MISSING for Done: one definition stated at the top of the paper and a single lemma connecting regret and Fisher-norm error (local quadratic equivalence KL ~ 1/2 ||.||^2_I with constants on a ratio set), not yet written.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="46.5" customHeight="1" s="27">
       <c r="A10" s="29" t="n">
@@ -1259,12 +1267,12 @@
       </c>
       <c r="L10" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="M10" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve"> LITERATURE 25 Oct: the two-point KL bound is already Herrera-Marin arXiv 2609.38268 Thm 2.2 + Cor 2.3 (empty start, shared mu and kernel shape, any normalised shape incl. sums of exponentials; unrefereed). Re-derived and tested on K=1 (bound held in 12/12 configs, 2-7x loose). Novelty here must come from online-estimator regret or other directions (individual alpha_k, stationary start). REASSESSMENT 25 Oct: as written this problem (two-point bound) is prior art (Herrera-Marin Thm 2.2). Suggested replacement: (a) regret lower bound for sequential estimators &gt;= (d/2) log T + (1/2) log det I - O(1); (b) identifiability map / matching UPPER bound on lambda_min(I) for the K-dictionary. Neither is proved; literature on regret lower bounds for point processes not yet searched.</t>
+          <t> LITERATURE 25 Oct: the two-point KL bound is already Herrera-Marin arXiv 2609.38268 Thm 2.2 + Cor 2.3 (empty start, shared mu and kernel shape, any normalised shape incl. sums of exponentials; unrefereed). Re-derived and tested on K=1 (bound held in 12/12 configs, 2-7x loose). Novelty here must come from online-estimator regret or other directions (individual alpha_k, stationary start). REASSESSMENT 25 Oct: as written this problem (two-point bound) is prior art (Herrera-Marin Thm 2.2). Suggested replacement: (a) regret lower bound for sequential estimators &gt;= (d/2) log T + (1/2) log det I - O(1); (b) identifiability map / matching UPPER bound on lambda_min(I) for the K-dictionary. Neither is proved; literature on regret lower bounds for point processes not yet searched. 25 Oct 2026. PARTIAL: (i) path-term two-point bound TV(Q_theta,Q_theta') &lt;= TV(pi_theta,pi_theta') + sqrt(rho T u'I u/2) (thm B); (ii) minimax lower bound for ANY predictor sup_Theta0 E R_n &gt;= (d/2) ln(n/ln n) - O(1) conditional on a uniformity hypothesis (U) (box_cost_and_lower_bound.md, Prop LB) matching the upper bound (d/2) ln T + C in the leading constant; (iii) non-consistency at eps=c/T for every k (problem11_observed_information.md, Thm NC, K=1). Upper-vs-lower comparison: leading constant d/2 matches (fixed eps); eps-dependence of the additive constant: upper O(eps^-2 ln 1/eps) (proof artefact), lower bound has no eps-explicit form; (U) unproved. MISSING for Done: the comparison table in eps, mu, T and an eps-explicit lower bound for eps = eps(n) -&gt; 0.</t>
         </is>
       </c>
     </row>
@@ -1845,10 +1853,14 @@
       </c>
       <c r="L20" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M20" s="33" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="M20" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026. PARTIAL: the simulation scripts exist and have been run (code/p5_*.py regret slopes: E R_n - ln T flat in eps, slope ~0.9 vs d/2 = 1 for K=1, ~1.3 vs 1.5 for K=2; code/p14_*.py tracking; code/p11_obs_info.py observed information; code/p13*.py from the other session), with tables in the notes. MISSING for Done: plots of error and regret versus T for several eps with fitted slopes compared with theory (no figures have been produced; the numbers are in tables only).</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="60" customHeight="1" s="27">
       <c r="A21" s="29" t="n">
@@ -2012,10 +2024,14 @@
       <c r="K23" s="29" t="n"/>
       <c r="L23" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M23" s="33" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="M23" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026. PARTIAL: literature_crosscheck.md, literature_search_report.md, novelty_reassessment.md (Herrera-Marin I/II, Jaisson-Rosenbaum, CIR drift papers, Hall-Willett, Yang et al., Piggott-Solo abstract only, Anne-Lu-Yu-Zhou 2026) with overlap-risk updates on the Literature sheet. MISSING for Done: 'difference from' statements for each core paper written as final text, and full-text reading of Piggott-Solo (closed access).</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="60" customHeight="1" s="27">
       <c r="A24" s="29" t="n">

</xml_diff>

<commit_message>
Problem 6: epsilon-explicit regret bound, potential-defect lemma, negative-moment lemma, simulations (K=1,2,3, k0<=1), tracker note
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1089,7 +1089,7 @@
       </c>
       <c r="M7" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. PARTIAL (problem05_E5_expected_regret.md, theoremR_proof_complete.md, K2_regret_chain.md, box_cost_and_lower_bound.md): Theorem R gives E R_T &lt;= (1/2 + O(delta+eta)) d ln T + C with C = O(mu d ln(1/(eps delta)) / (beta eps^2 delta^2)) (order only, K=1; general K with the tangent information level lambda_*/2); burn-in is ~1/eps^2 events (~1/(beta eps) in time units), not 1/(mu eps); no C log(1/eps) term visible in time units (leading term d/2 ln T + 1/2 ln det I with det I bounded for k0&gt;1). MISSING for Done: every constant of the theorem written as an explicit function of (eps, mu, K, beta-grid); the eps-dependence of C is an order, not a proved sharp rate.</t>
+          <t> 25 Oct 2026. PARTIAL (problem05_E5_expected_regret.md, theoremR_proof_complete.md, K2_regret_chain.md, box_cost_and_lower_bound.md): Theorem R gives E R_T &lt;= (1/2 + O(delta+eta)) d ln T + C with C = O(mu d ln(1/(eps delta)) / (beta eps^2 delta^2)) (order only, K=1; general K with the tangent information level lambda_*/2); burn-in is ~1/eps^2 events (~1/(beta eps) in time units), not 1/(mu eps); no C log(1/eps) term visible in time units (leading term d/2 ln T + 1/2 ln det I with det I bounded for k0&gt;1). MISSING for Done: every constant of the theorem written as an explicit function of (eps, mu, K, beta-grid); the eps-dependence of C is an order, not a proved sharp rate. 25 Oct 2026 (later), problem06_epsilon_explicit.md sections 9-14; code/p6_scaling.cs, p6_run.sh, p6_run2.sh, p6_analyze.py, p6_analyze2.py. RESULTS (K=1, mu=beta=1 unless stated): (1) E R_T - ln T is O(1) uniformly in eps in time units (-2.2,-1.5,-1.2,-2.9 for eps=0.3,0.1,0.03,0.01), so the eps^-2 ln(1/eps) in C is a proof artefact; in event units the constant is c_time - ln(mu/eps), which is where C log(1/eps) comes from. (2) Start cost is exactly P_0/2 = (rho_0/2)[eps Dmu^2/mu + (mu/eps)(Dalpha/beta)^2] (12.5 measured vs 12.0 at eps=0.01). (3) Lemma 6.4: tr X = ln det ratio + def, def &lt;= (tr X)^2, removes the leverage condition and the event count in the early phase; measured sum of def is O(1) (0.05-1.4) against 5.7e5 events at eps=0.01. (4) Burn-in measured: T_exit(0.25) ~ 2/(beta eps delta^2) (mixing-limited), flat in mu, not (k0-1)/(mu eps). (5) K=2 constant flat in eps (-6.0,-6.1,-5.7) but slope 1.2-1.3 &lt; 1.5 at T=3e4; K=3 not asymptotic; k0&lt;=1 slope 1 holds numerically with a larger constant. Theorem 6 (K=1, k0&gt;1) written with explicit constants up to hypothesis (D): D_early = O(d^2 ln^2(1/eps)). MISSING for Done: [superseded by the third pass below] 25 Oct 2026 (third pass, sections 15-18 of problem06_epsilon_explicit.md; code/p6_moments.cs, p6_chat.py, p6_tangent_det.py, p6_run3.sh). RESOLVED: (a) Lemma D1, negative moments E lam^-q &lt;= prod c_p, c_p = eps r/(mu-(p+1)B n^2/2), finite iff q &lt; k_eff = 2mu/(B n^2), proved for every K, matches simulation in 23/23 cases. (b) Prop D3: early-window regret handled by Prop 1 stopped at N_e plus Lemma D2 (E g'F^-1 g &lt;= 2(1+kappa^2) c+ E tr X), so no bad-gap count and no sup D; measured E X &lt;= P_0 + E G in 8/8 runs. (c) Prop D4: D_early = O(eps^a), a &lt; (k_eff-1)/2, proved for K=1, k0&gt;1, scaled prior (measured exponent 1.09); hypothesis (D) removed for that case. K&gt;=2: D1-D3 carry over, but the single-scale leverage constant grows like 1/eps (K=2: 72,157,461,1329 for eps=.3,.1,.03,.01), so D4 needs a mode-adapted bound (open); constants tabulated for K=2,3 (ln det I bracket: K=2 in [-4.63,-2.74], K=3 in [-9.1,-6.87]). k0&lt;=1: det I = (C eps^(k0-1) - 1)/beta^2 (k0&lt;1), (ln(1/eps)-1)/beta^2 (k0=1), so a genuine ((1-k0)/2) ln(1/eps) term appears in time units; D1 fails for k0&lt;=1. STILL OPEN: D4 for K&gt;=2 (mode-adapted leverage), for k0&lt;=1, and for a fixed (unscaled) prior; explicit burn-in constant for K&gt;=2; conservative universal constants c_1, C_1 of (H3).</t>
         </is>
       </c>
     </row>
@@ -1682,10 +1682,14 @@
       <c r="K17" s="29" t="n"/>
       <c r="L17" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M17" s="33" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M17" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026. problem16_kl_pseudotruth.md; code/p16/ (sim16.c, p16lib.py, t1..t7.py). Theorem 16 [P, draft, not independently verified]: under finite rate and E[lam*(1+|a|^2)]&lt;inf, L(theta)=E[lam* log(lam*/lam_theta)-lam*+lam_theta] is convex, strictly convex for distinct beta_k (linear independence of exponentials on a gap), coercive on the cone, so a unique theta-dagger exists on Theta_eps and on the cone; KKT: dL/dmu=E[1-lam*/lam]=rho_0, dL/dalpha_k=E[S_k(1-lam*/lam)]=rho_k-kappa/beta_k. Rate matching (new): mu-dagger=(1-n-dagger)Lambda* minus multiplier terms, so n(theta-dagger)&lt;1 automatically and the constraint n&lt;=1-eps is active iff the unconstrained immigrant share mu/Lambda* &lt; eps; when active mu-dagger=eps*Lambda*-kappa(1-eps). Quasi-MLE converges a.s. to theta-dagger. Numerics (power-law truth n*=0.8,0.95, K=1..4): rate matching to 4 digits, unique minimiser from several starts, KKT/kappa identities hold under active constraint, error of QMLE ~T^-1/2, Newton-decrement bound never violated. Found: n(theta-dagger)&lt;n*, increasing with K (0.46,0.62,0.70,0.73 at n*=0.8) - input to Problem 18. KL and quadratic surrogate differ by only 0.1-0.3% in these examples, so the advantage is structural not numerical. NOT proved: explicit strong-convexity constant, sandwich variance, a priori mu-dagger&gt;mu_min. SECOND PASS 25 Oct 2026 (problem16_kl_pseudotruth.md sec. 8, code/p16/t8.py, t9.py): explicit strong-convexity constant Hess L &gt;= lam_lo*E[aa'/(Lambda*+sum beta_k S_k)^2] (certified, valid and non-vacuous in all runs, conservative by 17-300x, worse with K and n*); consistency of the QMLE written out; sandwich variance H^-1 J H^-1 with J=H+misspecification terms, reproduced numerically (naive H^-1/T underestimates var(mu) by 40%, sandwich by 17%; equal in the well-specified control); CLT tagged P* (needs mixing). Still open: an a priori proof that mu-dagger&gt;mu_min (the natural bounds are vacuous; only the a-posteriori convexity certificate holds), active-constraint limit law. Replaces the earlier 'NOT proved' list except those two items. THIRD PASS 25 Oct 2026 (sec. 9, code/p16/t10.py, t11.py, t12.py): closed the last two open items. (i) A priori lower bound mu-dagger &gt;= mu_0, mu_0 = sup{mu: min_{alpha in A_eps} E[lam*/(mu+alpha'S)] &gt;= 1} [P], computable from the data law alone; non-vacuous in all runs (Phi(0)=1.06-1.63) but conservative 2-7x (mu_0~0.28 vs mu-dagger 1.55 at K=3, eps=0.05). (ii) Limit law with active constraints [P*]: sqrt(T)(theta-hat - theta-dagger) -&gt; V(V'HV)^-1 V'Z, rank d-|active|; tested K=2, n&lt;=0.5 active: var(mu) 3.41e-3 empirical vs 3.45e-3 formula (population J), corr -0.209 vs -0.210; unconstrained sandwich overstates 5x. Remaining caveats: CLT needs mixing (P*), strict complementarity assumed, batch-means J is 17-27% low at B=20.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="33" customHeight="1" s="27">
       <c r="A18" s="29" t="n">

</xml_diff>

<commit_message>
Problem 8: regret defined once (KL = expected log-loss regret), identity/sandwich/averaged-iterate lemmas, Wilks comparator, simulations, LaTeX definition block
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1206,12 +1206,12 @@
       </c>
       <c r="L9" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M9" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. PARTIAL: the notion used throughout is the log-loss (KL) regret of a predictive intensity, E R_n = KL(P_theta^(n) || Q^(n)) (box_cost_and_lower_bound.md B1), with pseudo-regret R_n = sum int lam* psi(lam_theta/lam*) &lt;= X_n pathwise; parameter error enters via the Fisher-norm quantities D_n = ||theta_{n+1}-theta*||^2_{F_n} (Lemma C1) and the tracking theorem (problem14_tracking_theorem.md); the lower bound passes from KL to MSE through mutual information (Prop LB). MISSING for Done: one definition stated at the top of the paper and a single lemma connecting regret and Fisher-norm error (local quadratic equivalence KL ~ 1/2 ||.||^2_I with constants on a ratio set), not yet written.</t>
+          <t> 25 Oct 2026. PARTIAL: the notion used throughout is the log-loss (KL) regret of a predictive intensity, E R_n = KL(P_theta^(n) || Q^(n)) (box_cost_and_lower_bound.md B1), with pseudo-regret R_n = sum int lam* psi(lam_theta/lam*) &lt;= X_n pathwise; parameter error enters via the Fisher-norm quantities D_n = ||theta_{n+1}-theta*||^2_{F_n} (Lemma C1) and the tracking theorem (problem14_tracking_theorem.md); the lower bound passes from KL to MSE through mutual information (Prop LB). MISSING for Done: one definition stated at the top of the paper and a single lemma connecting regret and Fisher-norm error (local quadratic equivalence KL ~ 1/2 ||.||^2_I with constants on a ratio set), not yet written. 25 Oct 2026 (later), problem08_regret_notion.md; latex/part2a_regret_notion.tex (added, included in hawkes_master.tex); code/p8_link.cs, p8_onestep.py, p8_run.sh, p8_analyze.py. DEFINITION FIXED: Reg_T = KL(P*_T || Q_T) = E r_T = E R_T (realised log-loss regret against the truth; R_T = int lam* psi(lam_hat/lam*) dt is its nonnegative pathwise version); all upper bounds bound E R, the lower bound is for the KL. LEMMAS: (identity) E r = E R via compensated martingale; (sandwich) Q_i/(2 c~+) &lt;= R_i &lt;= Q_i/(2 c~-^2), sharp 1/2 +- delta on R(delta); (regret =&gt; error) ||theta_bar - theta*||^2_J &lt;= 2 c~+ R_n for the information-weighted average, exact bias-variance identity; last iterate D_n=O(d) is NOT comparable to Reg_n ~ (d/2) ln T (same bound P_0+EG); hindsight regret = Reg + d/2 (Wilks), sign corrected. CHECKED: E r - E R within 1 se in 4000-replicate runs and in 28 single-gap cells; Lemma 8.1/8.2 no violations (4e5 grid points, ~1.9e6 gaps/run); sum R/(sum Q/2) = 0.95-1.01; averaged-iterate bound holds with margin &gt;=1.4; E D_n ~ d flat in n; hindsight-minus-truth = 1.0 (K=1), 1.4 (K=2) vs d/2. Audit table of existing theorems in section 8 (Hall-Willett regret is adversarial/dynamic, a different object). NOT COVERED: time-varying comparator (tracking), high-probability regret, converse for the last iterate. Remaining edit in existing text: replace the parenthetical after R_n in part2_regret.tex by a reference to Definition def:regret.</t>
         </is>
       </c>
     </row>
@@ -1743,10 +1743,14 @@
       </c>
       <c r="L18" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M18" s="33" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="M18" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026. problem17_online_convergence.md; code/p17/ (online17.c, lib17.py, w1,m1,m2,m3,trap,ev). Draft, not independently verified. Theorem 17A [P*]: projected online Newton (Fisher or observed-information preconditioner, exact F-norm projection) converges a.s. to the unique constrained KL pseudo-truth theta-dagger_Theta of Problem 16, active constraint included (ODE method with Markov noise + matrix gain; relies on cited Benveniste-Metivier-Priouret conditions, not re-verified). New exact facts: Lyapunov drift of ||theta-theta-dagger||^2_F is -v'(2Hbar - I_F)v with a favourable-sign multiplier term when the constraint binds; A = I_F^-1 H has eigenvalue exactly 1 at an interior theta-dagger. Theorem 17B/C [P*]: sqrt(n)(theta_n - theta-dagger) -&gt; N(0,Sigma), Lyapunov equation (A-1/2)Sigma+Sigma(A-1/2)'=Lambda* Ibar^-1 J Ibar^-1; with observed-information preconditioner Sigma = Lambda* H^-1 J H^-1 (batch sandwich) with no side condition; active constraint: same in the face subspace, n*dist to face -&gt; const (O(1/n)), projection active in a stable 3% of steps. Numerics (power-law truth n*=0.8, K=2, 600 replicates up to 1e5 events): n*Var matches prediction to 5-14% interior and 1-12% with active constraint (MC ~6%); n*MSE flat (rate 1/n); eigenvalues of I_F^-1 H in [0.97,1.002] in every example so EF=OI; OI corner-trapping found in 1/300 runs when mu_min=1e-3, none for EF or mu_min&gt;=0.1. MISSING for Done: self-contained proof of the Poisson-equation/regularity step, rigorous excursion bound for the distance to the face, degenerate (no strict complementarity) case, regret statement (Prop 17.4 is a conjecture), K&gt;2.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="46.5" customHeight="1" s="27">
       <c r="A19" s="29" t="n">

</xml_diff>

<commit_message>
Problem 9: Fisher-form two-point bound, matrix-covariance Bayes lower bound, eps-dependence (collapse in T*eps), comparison table, simulations
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1272,7 +1272,7 @@
       </c>
       <c r="M10" s="33" t="inlineStr">
         <is>
-          <t> LITERATURE 25 Oct: the two-point KL bound is already Herrera-Marin arXiv 2609.38268 Thm 2.2 + Cor 2.3 (empty start, shared mu and kernel shape, any normalised shape incl. sums of exponentials; unrefereed). Re-derived and tested on K=1 (bound held in 12/12 configs, 2-7x loose). Novelty here must come from online-estimator regret or other directions (individual alpha_k, stationary start). REASSESSMENT 25 Oct: as written this problem (two-point bound) is prior art (Herrera-Marin Thm 2.2). Suggested replacement: (a) regret lower bound for sequential estimators &gt;= (d/2) log T + (1/2) log det I - O(1); (b) identifiability map / matching UPPER bound on lambda_min(I) for the K-dictionary. Neither is proved; literature on regret lower bounds for point processes not yet searched. 25 Oct 2026. PARTIAL: (i) path-term two-point bound TV(Q_theta,Q_theta') &lt;= TV(pi_theta,pi_theta') + sqrt(rho T u'I u/2) (thm B); (ii) minimax lower bound for ANY predictor sup_Theta0 E R_n &gt;= (d/2) ln(n/ln n) - O(1) conditional on a uniformity hypothesis (U) (box_cost_and_lower_bound.md, Prop LB) matching the upper bound (d/2) ln T + C in the leading constant; (iii) non-consistency at eps=c/T for every k (problem11_observed_information.md, Thm NC, K=1). Upper-vs-lower comparison: leading constant d/2 matches (fixed eps); eps-dependence of the additive constant: upper O(eps^-2 ln 1/eps) (proof artefact), lower bound has no eps-explicit form; (U) unproved. MISSING for Done: the comparison table in eps, mu, T and an eps-explicit lower bound for eps = eps(n) -&gt; 0.</t>
+          <t> LITERATURE 25 Oct: the two-point KL bound is already Herrera-Marin arXiv 2609.38268 Thm 2.2 + Cor 2.3 (empty start, shared mu and kernel shape, any normalised shape incl. sums of exponentials; unrefereed). Re-derived and tested on K=1 (bound held in 12/12 configs, 2-7x loose). Novelty here must come from online-estimator regret or other directions (individual alpha_k, stationary start). REASSESSMENT 25 Oct: as written this problem (two-point bound) is prior art (Herrera-Marin Thm 2.2). Suggested replacement: (a) regret lower bound for sequential estimators &gt;= (d/2) log T + (1/2) log det I - O(1); (b) identifiability map / matching UPPER bound on lambda_min(I) for the K-dictionary. Neither is proved; literature on regret lower bounds for point processes not yet searched. 25 Oct 2026. PARTIAL: (i) path-term two-point bound TV(Q_theta,Q_theta') &lt;= TV(pi_theta,pi_theta') + sqrt(rho T u'I u/2) (thm B); (ii) minimax lower bound for ANY predictor sup_Theta0 E R_n &gt;= (d/2) ln(n/ln n) - O(1) conditional on a uniformity hypothesis (U) (box_cost_and_lower_bound.md, Prop LB) matching the upper bound (d/2) ln T + C in the leading constant; (iii) non-consistency at eps=c/T for every k (problem11_observed_information.md, Thm NC, K=1). Upper-vs-lower comparison: leading constant d/2 matches (fixed eps); eps-dependence of the additive constant: upper O(eps^-2 ln 1/eps) (proof artefact), lower bound has no eps-explicit form; (U) unproved. MISSING for Done: the comparison table in eps, mu, T and an eps-explicit lower bound for eps = eps(n) -&gt; 0. 25 Oct 2026 (later), problem09_lower_bound.md; latex/part2b_extensions.tex (Prop twopoint, Prop LBmat, Thm LBeps added); code/p9_bayes.cs, p9_run.sh, p9_run2.sh, p9_analyze.py. RESULTS (K=1): (1) Prop 9.0 two-point KL in Fisher form for exponential dictionaries, direction-resolved: (T/(2c+))u'Iu &lt;= KL &lt;= (T/(2c-^2))u'Iu; measured ratio 0.965-1.000 (delta&lt;=0.4 eps), always inside the bracket. (2) Prop 9.1: matrix-covariance Bayes lower bound sup Reg &gt;= ln|Theta0| + (d/2)ln(T/(2 pi e kappa)) + 0.5 ln det A; (U) is no longer a hypothesis: Newton satisfies it with A=N (tangent minorant), kappa_T ~ c ln T (measured kappa_eff ~ 1). (3) eps-dependence: over the stability band Theta0(eps) (alpha-width ~ eps) the Bayes regret collapses onto a function of x = T*eps alone (0.165+-0.01 at x=3 for eps from 0.3 to 0.003; ln x + const for large x), so minimax regret = ln(T eps) + O(1) for eps_T with T eps_T -&gt; inf; upper and lower bound have the same eps structure for k0&gt;1 up to 0.5 ln ln T + O(1); for k0&lt;1 the upper bound has the extra ((1-k0)/2) ln(1/eps) (needed to make the measured constant flat), the tangent minorant does not see it. (4) L_emp (Prop 9.1 with measured covariance) &lt;= Newton Bayes regret in 31/31 rows, gap 0.05-0.46; rigorous-form L_N within ~1 of the regret for eps 0.3..0.003; Bayes regret = Gaussian-experiment benchmark I_G (0.5 ln det(I + T S^1/2 I S^1/2)) minus 0.35 (uniform vs Gaussian prior entropy) at large x. CORRECTION: predicted (d-1)/2 plateau for T eps&lt;1 is wrong for the natural band (both directions switch off together). MISSING for Done: removal of the ln ln T (needs E D_n = O(d)); minorant of 1/lam capturing P(lam&lt;=2mu) ~ eps^k0 so the lower bound sees the k0&lt;1 term; K&gt;=2 simulations (propositions are K-general); uniformity of constants of Thm 9.3 over Theta0 written out.</t>
         </is>
       </c>
     </row>
@@ -1804,10 +1804,14 @@
       </c>
       <c r="L19" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M19" s="33" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M19" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026. problem18_bias_vs_K.md; code/p18/ (fd18.py, e2..e8.py). Draft, not independently verified. PROVED reductions: (i) n*-n-dagger = (mu-dagger - mu*)/Lambda* (rate matching, Problem 16); (ii) the surrogate pseudo-truth is the weighted L2 pole approximant of G(s)=int nu/(beta+s) on the imaginary axis with weight Lambda*/|1-G|^2 (Hawkes spectrum), so the bias is the DC value of the approximation error and can be computed deterministically for any K (matches the simulations of Problem 16 to 0.004). CONJECTURE 18.4 (numerically supported): b_K = kappa(eta,r) * n* (tau beta_1)^eta / Gamma(1+eta), beta_1 = beta_top r^-(K-1), i.e. geometric decay in K at rate eta*ln r; kappa ~0.43 at eta=1/2 (0.7 at eta=0.15), independent of n* and of criticality; exponent confirmed over 3 decades of beta_1 (ratios 0.32 per decade vs 10^-0.5); fixed range saturates at the truncation floor kappa*n_low(beta_min). Also: coarse grids overshoot (bias changes sign; best ratio for fixed K: r~17 at K=4, 8 at K=6, 6 at K=8); KL and surrogate biases agree within ~0.002 for K&gt;=3. NOT proved: the exponent eta and kappa&gt;0 (Wiener-Hopf/Newman-Stahl type problem for a geometric pole ladder), the discretization-floor law ~exp(-pi^2/ln r), general nu beyond the gamma form.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="46.5" customHeight="1" s="27">
       <c r="A20" s="29" t="n">

</xml_diff>

<commit_message>
Problem 19: simulation study (Ogata thinning), figures with bootstrap slope fits, burn-in and start-cost checks
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1865,12 +1865,12 @@
       </c>
       <c r="L20" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M20" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. PARTIAL: the simulation scripts exist and have been run (code/p5_*.py regret slopes: E R_n - ln T flat in eps, slope ~0.9 vs d/2 = 1 for K=1, ~1.3 vs 1.5 for K=2; code/p14_*.py tracking; code/p11_obs_info.py observed information; code/p13*.py from the other session), with tables in the notes. MISSING for Done: plots of error and regret versus T for several eps with fitted slopes compared with theory (no figures have been produced; the numbers are in tables only).</t>
+          <t> 25 Oct 2026. PARTIAL: the simulation scripts exist and have been run (code/p5_*.py regret slopes: E R_n - ln T flat in eps, slope ~0.9 vs d/2 = 1 for K=1, ~1.3 vs 1.5 for K=2; code/p14_*.py tracking; code/p11_obs_info.py observed information; code/p13*.py from the other session), with tables in the notes. MISSING for Done: plots of error and regret versus T for several eps with fitted slopes compared with theory (no figures have been produced; the numbers are in tables only). 25 Oct 2026 (later), problem19_simulation_study.md; figures/p19_*.png (5 figures); code/p19_sim.cs, p19_run.sh, p19_analyze.py, p19_thinning_check.py, p19_summary.txt. DONE: raw per-replicate runs (Ogata thinning, known mu, alpha, beta; ~1e9 events) for K=1 eps 0.3/0.1/0.03/0.01 (near and far start) and K=2 eps 0.3/0.1/0.03; sampler validated by time-rescaling (KS p 0.79-0.99). FITS (95% bootstrap CI): regret slope vs ln T contains d/2 in 10/10 runs (K=1: 0.95,0.96,1.10,1.08; K=2: 1.44,1.57,1.41 vs 1.5); raw MSE log-log slope -1 (inside for T eps &gt;= 700) and MSE*T/(I^-1)_jj = 1+-0.25; whitened error covariance eigenvalues ~(1,1), v'(TI)v ~ chi2_2; E D_n = 1.85-2.17 (d=2), 2.9-3.2 (d=3); burn-in T_exit ~ 1/eps, fits information form 1.4 max_j (I^-1)_jj/(delta theta_j)^2 within 0.85-1.23 for all 10 runs (K=2: middle tier binds); far-start excess matches (P0far-P0near)/2 (10.66+-2.06 vs 10.05 at eps=0.01). LIMITS: clip not exact F-projection; eps=0.01 only T eps=180 (not asymptotic: error slopes -1.6/-1.3, constant drift +0.8); K=3 and k0&lt;=1 not run here; slope CIs ~ +-0.13 (K=1), +-0.2 (K=2). Real-data and baselines are Problems 20 and 21.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Problem 21: baselines (batch MLE, Hall-Willett-type mirror descent, Solo-type EWLS) on identical simulated paths: error, regret, CPU tables
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1983,10 +1983,14 @@
       </c>
       <c r="L22" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M22" s="33" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="M22" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026, problem21_baselines.md; code/p21_baselines.cs, p21_run.sh, p21_analyze.py, p21_summary.txt; figures/p21_*.png. SIMULATED HALF DONE: batch MLE (constrained, same box), Hall-Willett-type mirror descent (log mirror map on theta, const / 1/sqrt(i) / 1/i steps, 6 step sizes) and Solo-type fixed-gain EWLS (rho = 1, 1-1/2000, 1-1/200), all on identical paths (K=1 eps 0.3/0.1/0.03, K=2 eps 0.1), error + regret + CPU. RESULTS at n=1e5: ours e_n = batch MLE to 0.01-0.02 (1.78/1.80, 2.16/2.15, 1.86/1.87, K=2 4.08/4.09; target d); ours better than batch at small n (n=95: 0.83 vs 4.50). Solo-type rho=1 inefficient by the predicted factor tr(I B^-1 C B^-1)/d = 1.22/1.50/1.75/1.38 (predicted 2.45/2.99/3.50/4.15, measured 2.48/3.66/3.08/4.92), fixed gain has non-vanishing error (e_n ~ n, linear regret). HW-type with eta0 tuned on the truth is 4.5-28x above d (no curvature, condition number ~ eps^-2); default step diverges. COST: ours 1.6 us/event (K=1), 2.3 (K=2), constant; mirror descent 0.08/0.10; EWLS 0.42/0.59; batch refit 0.33-0.4 us per data event per refit (linear in n), keeping batch current after every event ~ 1.1-1.3e4 us/event at n=2e5 (6000-7000x ours). CAVEATS: HW and Solo are adaptations (HW designed for intensity tracking with sqrt T regret, Solo read as abstract only; fixed gain is a feature for tracking, not static estimation). MISSING for Done: real-data comparison (needs tick data, Problem 20); protocol fixed (same stream, same box, distance to full-sample MLE and held-out log-loss replace e_n).</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="46.5" customHeight="1" s="27">
       <c r="A23" s="29" t="n">
@@ -2036,12 +2040,12 @@
       <c r="K23" s="29" t="n"/>
       <c r="L23" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M23" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. PARTIAL: literature_crosscheck.md, literature_search_report.md, novelty_reassessment.md (Herrera-Marin I/II, Jaisson-Rosenbaum, CIR drift papers, Hall-Willett, Yang et al., Piggott-Solo abstract only, Anne-Lu-Yu-Zhou 2026) with overlap-risk updates on the Literature sheet. MISSING for Done: 'difference from' statements for each core paper written as final text, and full-text reading of Piggott-Solo (closed access).</t>
+          <t> 25 Oct 2026. PARTIAL: literature_crosscheck.md, literature_search_report.md, novelty_reassessment.md (Herrera-Marin I/II, Jaisson-Rosenbaum, CIR drift papers, Hall-Willett, Yang et al., Piggott-Solo abstract only, Anne-Lu-Yu-Zhou 2026) with overlap-risk updates on the Literature sheet. MISSING for Done: 'difference from' statements for each core paper written as final text, and full-text reading of Piggott-Solo (closed access). 25 Oct 2026 (second pass). literature_difference_statements.md: one 'difference from' paragraph for each core paper (Herrera-Marin I and II, Hall-Willett, Yang et al., Piggott-Solo + Pasha-Solo) and for the papers that bear on Problems 16-18 (Rong-Nair 2602.20795, Wei-Zhu-Zhang-Xie 2006.09439, Spreij 1986/1991), plus a related-work draft. Each paragraph states its access level. KEY FINDINGS: the generic KL pseudo-truth/sandwich content of Problem 16 is anticipated in batch form by Wei et al. 2021; the LS pseudo-truth and a CLT without mixing by Rong-Nair 2026 (possible overlap with Prop 18.2); well-specified recursive estimation by Spreij. STILL MISSING: full texts of Piggott-Solo and Pasha-Solo (abstract only), Spreij scans (image-only, not OCRed), Herrera-Marin II Thm 3.1, end of Rong-Nair. Statement text should be rechecked against those before submission.</t>
         </is>
       </c>
     </row>
@@ -2093,10 +2097,14 @@
       <c r="K24" s="29" t="n"/>
       <c r="L24" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M24" s="33" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="M24" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026. literature_unverified_items.md. Searched/fetched all listed items. Zhang 2023: no matching paper found (identity unresolved). Wang 2023 = Technometrics online CUSUM change-point detector (not an estimator). Online EM for Hawkes: none found; Zhou-Zha-Song is batch ADMM; Lemonnier-Vayatis attribution unconfirmed. Cartea-Cohen-Labyad: batch LS gradient sampling, no regret. Bacry et al.: no misspecification paper located. Citation trees screened by titles (Hall-Willett via Semantic Scholar: 64; Yang et al. via OpenAlex: 26; a second Semantic Scholar query hit HTTP 429). Found beyond the list: Wei-Zhu-Zhang-Xie AISTATS 2021 (KL pseudo-truth, QMLE sandwich), Rong-Nair 2026 (LS pseudo-truth, CLT), Spreij 1986/1991 (recursive estimators for counting processes), Pasha-Solo CDC 2019 (fixed-gain), Lima 2021 (eps-margin stabilisation). Overlap-risk column updated. UNRESOLVED: Zhang 2023, online EM, full texts of Spreij/Solo papers.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M24"/>
@@ -3469,7 +3477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="26" min="1" max="1"/>
@@ -3760,7 +3768,7 @@
       </c>
       <c r="H7" s="32" t="inlineStr">
         <is>
-          <t>Reading: abstract read 25 Oct 2026 (via OpenAlex); full text NOT obtained. Fixed-gain exponentially weighted least squares on a Laguerre basis, non-negativity preserving, two time scales, simulations; abstract states no regret bound or near-critical analysis. See literature_search_report.md.</t>
+          <t>Reading: abstract read 25 Oct 2026 (via OpenAlex); full text NOT obtained. Fixed-gain exponentially weighted least squares on a Laguerre basis, non-negativity preserving, two time scales, simulations; abstract states no regret bound or near-critical analysis. See literature_search_report.md. Also: Pasha and Solo, CDC 2019, Adaptive Estimation of a Vector Point Process Model (abstract: fixed-gain adaptive estimator on the instantaneous likelihood, non-negativity constraints, genomic application). Full texts of both still not obtained.</t>
         </is>
       </c>
     </row>
@@ -3795,12 +3803,12 @@
       </c>
       <c r="G8" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H8" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Read 25 Oct 2026 (first ~200k of 213k characters of the HTML). Batch LS on a prescribed unit-mass basis; pseudo-true parameters via the LS contrast (Section 5.3, Thm 15) and CLTs under correct spec (Thm 17) and misspecification (Thm 21) by a martingale route with no mixing; numerics P=1..5 vs a sum-of-exponentials truth (no rate, no power law). No KL, no online, no proof of Gamma*&lt;1. May anticipate Prop 18.2 and the surrogate rate matching; route for the CLT item. See literature_difference_statements.md.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4290,7 @@
       </c>
       <c r="H20" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Searched 25 Oct 2026 (4 queries): no matching 2023 paper found; identity of the cited work unresolved. Wang et al. 2023 (Technometrics 65(1):44-56) is an online recursive CUSUM change-point detector, not an estimator. See literature_unverified_items.md.</t>
         </is>
       </c>
     </row>
@@ -4319,12 +4327,12 @@
       </c>
       <c r="G21" s="29" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H21" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Searched 25 Oct 2026: no online EM for Hawkes found. Zhou-Zha-Song (AISTATS 2013, PMLR 31:641-649) is batch ADMM (ADM4). Lemonnier-Vayatis attribution NOT confirmed (search returned Lemonnier-Scaman-Kalogeratos, low-rank large-scale inference).</t>
         </is>
       </c>
     </row>
@@ -4361,12 +4369,12 @@
       </c>
       <c r="G22" s="29" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H22" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Searched 25 Oct 2026: Cartea-Cohen-Labyad (2111.10637) is a batch gradient method for the least-squares contrast (adaptive stratified sampling of the gradient); no regret/online/misspecification in the abstract. No Bacry et al. misspecification paper located.</t>
         </is>
       </c>
     </row>
@@ -4403,12 +4411,12 @@
       </c>
       <c r="G23" s="29" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H23" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Screened 25 Oct 2026 by titles: Hall-Willett tree 64 entries (Semantic Scholar), Yang et al. tree 26 entries (OpenAlex); second Semantic Scholar query rate-limited. Found: Pasha-Solo 2019, Lima 2021 (eps-margin stabilisation of parametric Hawkes MLE), Ghassemi et al. 2022 (online mixtures of MHP), Jaffard et al. 2024 (learning rule for Hawkes networks), Xu et al. 2018. None on misspecification or the near-critical ratio by title.</t>
         </is>
       </c>
     </row>
@@ -4652,10 +4660,346 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="30" customHeight="1" s="27">
-      <c r="B31" s="42" t="inlineStr">
-        <is>
-          <t>Details come from my research summary of 24 Oct 2026. Re-check every claim against the primary source before citing. Herrera-Marín papers are unrefereed arXiv preprints. Overlap risk is my judgement. Updated 25 Oct 2026: rows 7 and 17 corrected, rows 24-29 added from literature_search_report.md; most new entries were read only in part (see Read status).</t>
+    <row r="30" ht="46.5" customHeight="1" s="27">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>Goodness-of-Fit Test for Mismatched Self-Exciting Processes</t>
+        </is>
+      </c>
+      <c r="C30" s="30" t="inlineStr">
+        <is>
+          <t>Wei, Zhu, Zhang, Xie, AISTATS 2021 (PMLR 130:1243-1251)</t>
+        </is>
+      </c>
+      <c r="D30" s="30" t="inlineStr">
+        <is>
+          <t>arXiv 2006.09439</t>
+        </is>
+      </c>
+      <c r="E30" s="29" t="inlineStr">
+        <is>
+          <t>16, 17</t>
+        </is>
+      </c>
+      <c r="F30" s="30" t="inlineStr">
+        <is>
+          <t>QMLE theory under misspecification: KL pseudo-truth by concavity (Prop 2), a.s. convergence (Lemma 1), sandwich covariance.</t>
+        </is>
+      </c>
+      <c r="G30" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H30" s="32" t="inlineStr">
+        <is>
+          <t>Read 25 Oct 2026 (about 100k of 136k characters of ar5iv). Piecewise-constant triggering, batch, near-critical not analysed. Anticipates the generic part of Theorem 16 / Prop 16.7; not the exponential dictionary with stability set, rate matching, active constraint, online.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="46.5" customHeight="1" s="27">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B31" s="31" t="inlineStr">
+        <is>
+          <t>Recursive parameter estimation for counting processes with linear intensity; Recursive approximate maximum likelihood estimation for a class of counting process models</t>
+        </is>
+      </c>
+      <c r="C31" s="30" t="inlineStr">
+        <is>
+          <t>Spreij, Stochastics 18 (1986) 277-312; J. Multivariate Anal. 39 (1991) 236-245</t>
+        </is>
+      </c>
+      <c r="D31" s="30" t="inlineStr">
+        <is>
+          <t>CWI R 8513 / ir.cwi.nl pub 2491, 6311; staff.fnwi.uva.nl/p.j.c.spreij</t>
+        </is>
+      </c>
+      <c r="E31" s="29" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="F31" s="30" t="inlineStr">
+        <is>
+          <t>Recursive MLE-type estimators for intensities linear in theta: consistency and asymptotic normality by stochastic Lyapunov functions.</t>
+        </is>
+      </c>
+      <c r="G31" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H31" s="32" t="inlineStr">
+        <is>
+          <t>Abstract-level only (25 Oct 2026); the scans are image-only and were not OCRed. Likely anticipates the well-specified recursive consistency/CLT of Problem 17; misspecification, active constraint, regret, near-critical not known to be covered. Read first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="46.5" customHeight="1" s="27">
+      <c r="A32" s="29" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>Adaptive Estimation of a Vector Point Process Model</t>
+        </is>
+      </c>
+      <c r="C32" s="30" t="inlineStr">
+        <is>
+          <t>Pasha and Solo, CDC 2019, pp. 2904-2909</t>
+        </is>
+      </c>
+      <c r="D32" s="30" t="inlineStr">
+        <is>
+          <t>IEEE Xplore (dblp conf/cdc/PashaS19)</t>
+        </is>
+      </c>
+      <c r="E32" s="29" t="inlineStr">
+        <is>
+          <t>13, 15, 21</t>
+        </is>
+      </c>
+      <c r="F32" s="30" t="inlineStr">
+        <is>
+          <t>Fixed-gain adaptive estimator on the instantaneous likelihood of a log-intensity model with non-negativity constraints.</t>
+        </is>
+      </c>
+      <c r="G32" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H32" s="32" t="inlineStr">
+        <is>
+          <t>Abstract only (25 Oct 2026). Companion of the Piggott-Solo row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="46.5" customHeight="1" s="27">
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="inlineStr">
+        <is>
+          <t>Fine-Grained epsilon-Margin Closed-Form Stabilization of Parametric Hawkes Processes</t>
+        </is>
+      </c>
+      <c r="C33" s="30" t="inlineStr">
+        <is>
+          <t>Lima, arXiv, May 2021</t>
+        </is>
+      </c>
+      <c r="D33" s="30" t="inlineStr">
+        <is>
+          <t>arXiv 2105.03800</t>
+        </is>
+      </c>
+      <c r="E33" s="29" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="F33" s="30" t="inlineStr">
+        <is>
+          <t>Uses an epsilon margin on the stability condition to stabilise parametric MLE.</t>
+        </is>
+      </c>
+      <c r="G33" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H33" s="32" t="inlineStr">
+        <is>
+          <t>Abstract only (25 Oct 2026). Anticipates the device n&lt;=1-eps, not the analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="46.5" customHeight="1" s="27">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>Gradient-based estimation of linear Hawkes processes with general kernels</t>
+        </is>
+      </c>
+      <c r="C34" s="30" t="inlineStr">
+        <is>
+          <t>Cartea, Cohen, Labyad, arXiv Nov 2021</t>
+        </is>
+      </c>
+      <c r="D34" s="30" t="inlineStr">
+        <is>
+          <t>arXiv 2111.10637</t>
+        </is>
+      </c>
+      <c r="E34" s="29" t="inlineStr">
+        <is>
+          <t>5, 21</t>
+        </is>
+      </c>
+      <c r="F34" s="30" t="inlineStr">
+        <is>
+          <t>Adaptive stratified sampling of the least-squares gradient for large datasets.</t>
+        </is>
+      </c>
+      <c r="G34" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H34" s="32" t="inlineStr">
+        <is>
+          <t>Abstract only (25 Oct 2026). Batch LS, no regret.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="46.5" customHeight="1" s="27">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B35" s="31" t="inlineStr">
+        <is>
+          <t>Online recursive CUSUM for Hawkes networks (Wang et al.)</t>
+        </is>
+      </c>
+      <c r="C35" s="30" t="inlineStr">
+        <is>
+          <t>Wang, Xie, Xie, Cuozzo, Mak, Technometrics 65(1):44-56 (2023)</t>
+        </is>
+      </c>
+      <c r="D35" s="30" t="inlineStr">
+        <is>
+          <t>DOI 10.1080/00401706.2022.2054862</t>
+        </is>
+      </c>
+      <c r="E35" s="29" t="inlineStr">
+        <is>
+          <t>14, 20</t>
+        </is>
+      </c>
+      <c r="F35" s="30" t="inlineStr">
+        <is>
+          <t>Online change-point detection for Hawkes networks.</t>
+        </is>
+      </c>
+      <c r="G35" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H35" s="32" t="inlineStr">
+        <is>
+          <t>Abstract only (25 Oct 2026). Detection, not estimation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="46.5" customHeight="1" s="27">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>Provable local learning rule by expert aggregation for a Hawkes network</t>
+        </is>
+      </c>
+      <c r="C36" s="30" t="inlineStr">
+        <is>
+          <t>Jaffard, Vaiter, Muzy, Reynaud-Bouret, AISTATS 2024</t>
+        </is>
+      </c>
+      <c r="D36" s="30" t="inlineStr">
+        <is>
+          <t>arXiv 2304.08061</t>
+        </is>
+      </c>
+      <c r="E36" s="29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F36" s="30" t="inlineStr">
+        <is>
+          <t>Hawkes network used as a classifier learned by expert aggregation; local regret bounds.</t>
+        </is>
+      </c>
+      <c r="G36" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H36" s="32" t="inlineStr">
+        <is>
+          <t>Abstract only (25 Oct 2026). Not parametric estimation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="46.5" customHeight="1" s="27">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B37" s="31" t="inlineStr">
+        <is>
+          <t>Online Learning for Mixture of Multivariate Hawkes Processes</t>
+        </is>
+      </c>
+      <c r="C37" s="30" t="inlineStr">
+        <is>
+          <t>Ghassemi et al., ICAIF 2022</t>
+        </is>
+      </c>
+      <c r="D37" s="30" t="inlineStr">
+        <is>
+          <t>arXiv 2208.07961</t>
+        </is>
+      </c>
+      <c r="E37" s="29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F37" s="30" t="inlineStr">
+        <is>
+          <t>Streaming mixtures of MHP.</t>
+        </is>
+      </c>
+      <c r="G37" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H37" s="32" t="inlineStr">
+        <is>
+          <t>Title/abstract-level only (25 Oct 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1" s="27">
+      <c r="B38" s="42" t="inlineStr">
+        <is>
+          <t>Details come from my research summary of 24 Oct 2026. Re-check every claim against the primary source before citing. Herrera-Marín papers are unrefereed arXiv preprints. Overlap risk is my judgement. Updated 25 Oct 2026: rows 7 and 17 corrected, rows 24-29 added from literature_search_report.md; most new entries were read only in part (see Read status). Updated again 25 Oct 2026 (second pass): rows 25-32 added; Rong-Nair risk raised to High; the four to-check rows filled in (literature_unverified_items.md).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Problem 20: real-data check on Deribit BTC option trades (no NSE tick data available): n_hat(t), dictionary selection, misspecification, online vs batch
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1028,7 +1028,7 @@
       </c>
       <c r="M6" s="33" t="inlineStr">
         <is>
-          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled). CLOSED 25 Oct (Done): Theorem HP (problem05_07_closure.md): with prob &gt;= 1-6e^-x-P(E^c), R_n &lt;= psi_max(2 i0+3x) + 4[D0' + x/theta + G_n(x)]; plus expected-regret Thm R (sharp constant). Assumptions: known compact convex Theta_c, leverage event, Assumption M (certified K=1) / lambda_L (K&gt;=2). FINAL AUDIT 25 Oct (final_audit.md): fixed constant in Lemma E5c (xbar = lbar m/(c^- mu*), not c^+), replaced loose general-K Lemma E1 by the exact Z_c identity; K=2 pathwise Newton/martingale inequalities verified (code/p5_k2_pathwise_check.py). STRENGTHENED 25 Oct: (1) theoremR_proof_complete.md writes every step of the expected-regret theorem (assembly needs only predictable good-gap indicators + one per-time failure bound H3); (2) information level without Assumption M via the tangent minorant: lambda_*/2 ~ 0.013 for the K=2 example vs ~1e-6 before.</t>
+          <t>25 Oct 2026. problem05_online_newton.md; code/p5_*.py. First pass, K=1 only. Proposition 1 (rigorous, short): for the unprojected Fisher-scoring/online-Newton update, E&lt;g_i,v_i | past&gt; = E[v_i' dF_i v_i | past] exactly (first-event compensator identity), hence E R_n &lt;= ||th_1-th*||^2_{F_0} + E sum g_i' F_i^-1 g_i, no exp-concavity needed. Checked numerically (pathwise identity to 1e-13; expectation identity within SE; bound ~2x loose). Empirical: regret slope (d/2) in log n; E[R_n - log T_n] ~ flat in eps (-1.2,-2.3,-2.4,-2.8 for eps=.3,.1,.03,.01): no visible +C log(1/eps) in time units; apparent 0.5/eps burn-in cost was the prior term rho0*|th_1-th*|^2, vanishes with a weak prior. NOT proven: bound on G (needs leverage bound a'F^-1 a/lam = O(1) and local control, i.e. Problem 7), sharp constant 1/2 (needs localisation), projected algorithm (diag projection not non-expansive in F-norm; unprojected iterates exit Theta_eps in 55-85% of runs), K&gt;=2, high-probability version. Draft, not independently verified. UPDATE 25 Oct: problem05_fisher_concentration.md (K=1, oracle information): Lemma F1 var(int h(S_t)dt) &lt;= 2T Lip sqrt(m) sigma_S/gamma via the Problem-3 contraction; Lemma F2 two-interval bound J_T &gt;= (O/L) Q (exact, deterministic); Theorem F: J_T &gt;= (mT/4L) Q w.p. &gt;=1-2q for all T&gt;=T0=16 sigma_S/(rho gamma m^1.5 q) = O(1/(beta eps)), so Theorem-7 leverage assumptions hold w.h.p. given (L1). Numerics: variance bound holds with 500-1500x margin; pathwise leverage bound 0 violations in ~1300 checks; rigorous T0*gamma ~ 4e5 vs empirical ~20-50 (Chebyshev, 1e4x conservative). OPEN: circularity (L1 needs consistency which needs the information bound), Assumption M (pi-mass of bumps, numerical), exponential tails, projection, K&gt;=2. UPDATE 25 Oct (problem05_circularity.md): circularity avoided by design, not by a consistency bootstrap: compact box Theta_c known a priori + exact F-norm projection =&gt; (L1) holds deterministically (c+=max(mu_hi/mu*,al_hi/al*), c-=min(...)); Prop 1 survives projection (non-expansiveness in F-norm); leverage w.h.p. after T0=O(1/(beta eps)) via Theorem F. Numerics (K=1): R_n - log T_n between -4.4 and -0.5 in 24 configs, 0 non-expansiveness violations. Sketched only: stopping-time localisation of the w.h.p. event; burn-in term crude. OPEN: true bootstrap (c-&gt;1), K&gt;=2 (QP projection), a priori scale knowledge, exponential tails. UPDATE 25 Oct (problem05_bootstrap.md): TRUE BOOTSTRAP, K=1, two-stage, polynomial tails. Stage 1 with box constants: pathwise D_j &lt;= D0' - X - M + G (M martingale, E m^2 &lt;= (4/c-) E[v'dF v]); Doob L2 + Markov =&gt; P(sup D_j &gt;= 3x) &lt;= (1+16/c0-) Gamma/x, Gamma=O(d log T); with F &gt;= lam_T I this forces the iterates into R(delta) for t&gt;=T1 when delta^2 &gt;= 24(1+16/c0-)c0+ L Gamma/(q m lamQ rho*^2 T1) (T1 gamma ~ d log T1/delta^2). Stage 2: with c+-=1+-delta, A-&gt;1, B-&gt;0, psi-factor 2 -&gt; 1+O(delta): regret (d/2+o(1)) log T on the good event. Numerics: pathwise inequality margin 1e-14; E sum m^2/E X ~4; sup D_j &lt;=14; last exit time from R(delta) ~ 1-3/(delta^2 gamma), slope of E R_n in log T ~0.9 (target d/2=1). NOT proved: expected regret with sharp constant (needs exponential tails; bad event only ~1/T1), localisation bookkeeping, K&gt;=2, a-priori box. UPDATE 25 Oct (problem05_exponential_tails.md): exponential tails. E1 exact identities (eps*Lam_T = mu T + n M'_T - n dS; Poisson eq u=(s-ES)/gamma), verified 1e-14. E2 Lam_T tails exp(-eta^2 mu eps T/2n^2). E3 occupation functionals via Poisson equation + Freedman: P(int h &lt;= Tm/2) &lt;= 3 exp(-c T gamma), c=m^2 mu/(32 kappa^2 (1+eta) beta) ~3e-7 (empirical decay ~0.04-0.056 per unit T*gamma: bound valid but 1e5x pessimistic). E4 Newton martingale: with prob&gt;=1-e^-x, -M_t &lt;= X_t + x/theta for all t (theta=min(1/(2k1), c-/2.87)) so sup D_j &lt;= D0' + x/theta + G_n. Theorem C-exp: bootstrap with T1 = O((ln(1/q)+d log T)/(gamma delta^2)). NOT done: E5 (exp bound on G_n, martingale part of score sum) in detail; expected regret with sharp constant needs episode/restart argument (union bound would pay crude linear rate on [0, T_c ~ log T_n]); constants; K&gt;=2. REASSESSMENT 25 Oct (novelty_reassessment.md): C2's 'C log(1/eps)' should be made explicit: conjecture regret = (d/2) log T + (1/2) log det I(theta*;eps) + O(1) in time units, with (1/2) log det I ~ ((1-k)^+/2) log(1/eps), k=2*mu*m (m=mean lifetime). Exact K=1 slopes confirm the information side (0.40 for k0=0.2); the regret side is DISFAVOURED by a 100-rep test (k0=0.2, E[R - log T] = -3.44+-0.10 at eps=0.3 vs -3.19+-0.32 at eps=0.01, against +1.30 predicted); conjecture withdrawn from the headline. Caveat: the test starts at theta*, so it cannot probe a Bayes/redundancy lower-bound constant. E5 + EXPECTED REGRET 25 Oct (problem05_E5_expected_regret.md, K1_main_results.md): E5 PROVED (Lemmas E5a-d, Prop E5: G_n &lt;= (1+o(1)) logdet + o(1)x + B_X X w.p. &gt;= 1-4e^-x; pathwise inequalities checked, 0 violations in 1.4e6 gaps). Found+fixed a flaw in Theorem 7/Lemma 7c: 'gap leverage &lt;= xbar a.s.' cannot hold (depends on Exp(1) variable); truncation fixes it. Theorem R (K=1): E R_n &lt;= (1/2+O(delta+eta)) d ln T + C, C independent of n, via charging bad events to their own time (no episode union bound); PROVED MODULO Thm F-exp, Assumption M (numerical), known box, and unwritten optional-stopping across random restarts. Rate constants ~1e5 worse than observed. K&gt;=2 open. DEPENDENCIES 25 Oct (K1_completion.md): optional stopping closed (predictable good-gap indicators replace restarts); integrability in Thm F-exp closed; Assumption M closed for eps&lt;=eps_M via the Gamma comparator of Thm T (E_Gamma h = 0.164, 0.044 vs simulated 0.15, 0.05); C(eps)=O(mu d ln(1/(eps delta))/(beta eps^2 delta^2)) (order only). Still assumed: known box; K&gt;=2 open; constants conservative; Thm T itself is a proof outline with numerically verified estimates. ASSUMPTION M certified 25 Oct (thmT_explicit_constants.md): K=1, k0=2, mu=beta=1: m&gt;=0.0248 for eps&lt;=1e-4 (E_Gamma h = 0.164, 0.0444 minus TV&lt;=0.0196). EXTENSIONS 25 Oct (assumptionM_exact.md, box_cost_and_lower_bound.md, K2_regret_chain.md): (1) Assumption M certified by exact Fourier quadrature for K=1, eps&lt;=0.3, k0 in [0.6,4] (m&gt;=0.032); (2) box cost: polynomial in c+,1/c-, empirically ~s^2 at rho0=1 (prior effect), leading constant box-free; scale of mu* not learnable at eps=c/T; (3) K&gt;=2: chain carries over, Assumption M replaced by computable lambda_L (Thm FK), Thm R^(K) (K+1)/2 ln T + C_K, constants uninformative, K=2 slope ~1.3 vs 1.5 [N]; (4) minimax lower bound (d/2)ln n - O(ln ln n) for ANY predictor, conditional on uniformity (U). LaTeX master document: latex/hawkes_master.tex (not compiled). CLOSED 25 Oct (Done): Theorem HP (problem05_07_closure.md): with prob &gt;= 1-6e^-x-P(E^c), R_n &lt;= psi_max(2 i0+3x) + 4[D0' + x/theta + G_n(x)]; plus expected-regret Thm R (sharp constant). Assumptions: known compact convex Theta_c, leverage event, Assumption M (certified K=1) / lambda_L (K&gt;=2). FINAL AUDIT 25 Oct (final_audit.md): fixed constant in Lemma E5c (xbar = lbar m/(c^- mu*), not c^+), replaced loose general-K Lemma E1 by the exact Z_c identity; K=2 pathwise Newton/martingale inequalities verified (code/p5_k2_pathwise_check.py). STRENGTHENED 25 Oct: (1) theoremR_proof_complete.md writes every step of the expected-regret theorem (assembly needs only predictable good-gap indicators + one per-time failure bound H3); (2) information level without Assumption M via the tangent minorant: lambda_*/2 ~ 0.013 for the K=2 example vs ~1e-6 before. ATTRIBUTION (25 Oct 2026): the Fisher-preconditioned recursion of this problem is Spreij's AML recursion (1986/1991) applied to Hawkes; novelty of C1 lies in the log-loss regret analysis, the exact F-norm projection, the observed-information variant and the misspecified analysis, not the recursion. See refpapers_conclusions.md.</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="M18" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. problem17_online_convergence.md; code/p17/ (online17.c, lib17.py, w1,m1,m2,m3,trap,ev). Draft, not independently verified. Theorem 17A [P*]: projected online Newton (Fisher or observed-information preconditioner, exact F-norm projection) converges a.s. to the unique constrained KL pseudo-truth theta-dagger_Theta of Problem 16, active constraint included (ODE method with Markov noise + matrix gain; relies on cited Benveniste-Metivier-Priouret conditions, not re-verified). New exact facts: Lyapunov drift of ||theta-theta-dagger||^2_F is -v'(2Hbar - I_F)v with a favourable-sign multiplier term when the constraint binds; A = I_F^-1 H has eigenvalue exactly 1 at an interior theta-dagger. Theorem 17B/C [P*]: sqrt(n)(theta_n - theta-dagger) -&gt; N(0,Sigma), Lyapunov equation (A-1/2)Sigma+Sigma(A-1/2)'=Lambda* Ibar^-1 J Ibar^-1; with observed-information preconditioner Sigma = Lambda* H^-1 J H^-1 (batch sandwich) with no side condition; active constraint: same in the face subspace, n*dist to face -&gt; const (O(1/n)), projection active in a stable 3% of steps. Numerics (power-law truth n*=0.8, K=2, 600 replicates up to 1e5 events): n*Var matches prediction to 5-14% interior and 1-12% with active constraint (MC ~6%); n*MSE flat (rate 1/n); eigenvalues of I_F^-1 H in [0.97,1.002] in every example so EF=OI; OI corner-trapping found in 1/300 runs when mu_min=1e-3, none for EF or mu_min&gt;=0.1. MISSING for Done: self-contained proof of the Poisson-equation/regularity step, rigorous excursion bound for the distance to the face, degenerate (no strict complementarity) case, regret statement (Prop 17.4 is a conjecture), K&gt;2.</t>
+          <t> 25 Oct 2026. problem17_online_convergence.md; code/p17/ (online17.c, lib17.py, w1,m1,m2,m3,trap,ev). Draft, not independently verified. Theorem 17A [P*]: projected online Newton (Fisher or observed-information preconditioner, exact F-norm projection) converges a.s. to the unique constrained KL pseudo-truth theta-dagger_Theta of Problem 16, active constraint included (ODE method with Markov noise + matrix gain; relies on cited Benveniste-Metivier-Priouret conditions, not re-verified). New exact facts: Lyapunov drift of ||theta-theta-dagger||^2_F is -v'(2Hbar - I_F)v with a favourable-sign multiplier term when the constraint binds; A = I_F^-1 H has eigenvalue exactly 1 at an interior theta-dagger. Theorem 17B/C [P*]: sqrt(n)(theta_n - theta-dagger) -&gt; N(0,Sigma), Lyapunov equation (A-1/2)Sigma+Sigma(A-1/2)'=Lambda* Ibar^-1 J Ibar^-1; with observed-information preconditioner Sigma = Lambda* H^-1 J H^-1 (batch sandwich) with no side condition; active constraint: same in the face subspace, n*dist to face -&gt; const (O(1/n)), projection active in a stable 3% of steps. Numerics (power-law truth n*=0.8, K=2, 600 replicates up to 1e5 events): n*Var matches prediction to 5-14% interior and 1-12% with active constraint (MC ~6%); n*MSE flat (rate 1/n); eigenvalues of I_F^-1 H in [0.97,1.002] in every example so EF=OI; OI corner-trapping found in 1/300 runs when mu_min=1e-3, none for EF or mu_min&gt;=0.1. MISSING for Done: self-contained proof of the Poisson-equation/regularity step, rigorous excursion bound for the distance to the face, degenerate (no strict complementarity) case, regret statement (Prop 17.4 is a conjecture), K&gt;2. READ 25 Oct 2026 (refpapers_conclusions.md): the EF recursion is Spreij's AML recursion (Stochastics 1986; JMVA 1991) applied to the Hawkes regressor; his well-specified a.s. consistency (Lyapunov x'Q^-1 x, Lai-Wei growth condition, known coordinate box) and Cramer-Rao CLT are the A=I special case of Theorems 17A/17B, which are therefore NOT claimed as new. Still ours: misspecified target theta-dagger, drift matrix I_F^-1 H != I and the Lyapunov-equation limit law (+ Lemma 17.5), observed-information preconditioner, exact convex projection with a binding stability face / alpha_k=0, active-constraint limit law, regret. Overlap risk: High for the well-specified part, Low-Medium for the rest.</t>
         </is>
       </c>
     </row>
@@ -1926,10 +1926,14 @@
       </c>
       <c r="L21" s="32" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="M21" s="33" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="M21" s="33" t="inlineStr">
+        <is>
+          <t> 25 Oct 2026, problem20_real_data.md; code/p20_prep.py, p20_fit.cs, p20_run.sh, p20_analyze.py, p20_summary.txt; figures/p20_*.png. DATA: no NSE/Bank Nifty tick data exists (the Bank Nifty CSV is 1-minute option-chain snapshots; the 24 Oct directional-change events from minute bars are a different object). Real tick data that exist: Deribit BTC option trades, 5.41M trades -&gt; 4.77M distinct-ms events, 2024-11..2025-10 (market-data/btc-1y). Study done on BTC, window 13-20 UTC, 365 daily windows. RESULTS: dictionary beta=(0.1,1,10)/s chosen on held-out log-lik (improves monotonically with K: no finite dictionary correct; K=1 n_hat ranges 0.21-0.91 with beta). n_hat daily median 0.668 (10-90% 0.56-0.77, range 0.44-0.93), dispersion 5x its s.e., corr(n_hat, log activity)=+0.77, weekend 0.60 vs weekday 0.68; 2025-03-02 clustering jump (n_hat 0.93, low mu) vs 2025-10-10 baseline surge (mu 0.118, n_hat 0.80). Misspecification: median n_hat 0.50/0.55/0.67/0.66 for K=1/2/3/4, KS rejects K&lt;=3 on 98-100% of days, K=4 (100/s component) passes 85%. Online: growing-window = pooled batch MLE to 0.0025 (0.7565 vs 0.7590); forgetting estimators smooth the daily series (corr 0.34-0.50). Hourly fits too noisy (s.e. 0.045). OPEN: NSE/Bank Nifty tick data; baselines of Problem 21 on this stream (events.bin ready); near-critical regime not reached (n_hat 0.5-0.8).</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="46.5" customHeight="1" s="27">
       <c r="A22" s="29" t="n">
@@ -2045,7 +2049,7 @@
       </c>
       <c r="M23" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. PARTIAL: literature_crosscheck.md, literature_search_report.md, novelty_reassessment.md (Herrera-Marin I/II, Jaisson-Rosenbaum, CIR drift papers, Hall-Willett, Yang et al., Piggott-Solo abstract only, Anne-Lu-Yu-Zhou 2026) with overlap-risk updates on the Literature sheet. MISSING for Done: 'difference from' statements for each core paper written as final text, and full-text reading of Piggott-Solo (closed access). 25 Oct 2026 (second pass). literature_difference_statements.md: one 'difference from' paragraph for each core paper (Herrera-Marin I and II, Hall-Willett, Yang et al., Piggott-Solo + Pasha-Solo) and for the papers that bear on Problems 16-18 (Rong-Nair 2602.20795, Wei-Zhu-Zhang-Xie 2006.09439, Spreij 1986/1991), plus a related-work draft. Each paragraph states its access level. KEY FINDINGS: the generic KL pseudo-truth/sandwich content of Problem 16 is anticipated in batch form by Wei et al. 2021; the LS pseudo-truth and a CLT without mixing by Rong-Nair 2026 (possible overlap with Prop 18.2); well-specified recursive estimation by Spreij. STILL MISSING: full texts of Piggott-Solo and Pasha-Solo (abstract only), Spreij scans (image-only, not OCRed), Herrera-Marin II Thm 3.1, end of Rong-Nair. Statement text should be rechecked against those before submission.</t>
+          <t> 25 Oct 2026. PARTIAL: literature_crosscheck.md, literature_search_report.md, novelty_reassessment.md (Herrera-Marin I/II, Jaisson-Rosenbaum, CIR drift papers, Hall-Willett, Yang et al., Piggott-Solo abstract only, Anne-Lu-Yu-Zhou 2026) with overlap-risk updates on the Literature sheet. MISSING for Done: 'difference from' statements for each core paper written as final text, and full-text reading of Piggott-Solo (closed access). 25 Oct 2026 (second pass). literature_difference_statements.md: one 'difference from' paragraph for each core paper (Herrera-Marin I and II, Hall-Willett, Yang et al., Piggott-Solo + Pasha-Solo) and for the papers that bear on Problems 16-18 (Rong-Nair 2602.20795, Wei-Zhu-Zhang-Xie 2006.09439, Spreij 1986/1991), plus a related-work draft. Each paragraph states its access level. KEY FINDINGS: the generic KL pseudo-truth/sandwich content of Problem 16 is anticipated in batch form by Wei et al. 2021; the LS pseudo-truth and a CLT without mixing by Rong-Nair 2026 (possible overlap with Prop 18.2); well-specified recursive estimation by Spreij. STILL MISSING: full texts of Piggott-Solo and Pasha-Solo (abstract only), Spreij scans (image-only, not OCRed), Herrera-Marin II Thm 3.1, end of Rong-Nair. Statement text should be rechecked against those before submission. UPDATE 25 Oct 2026: Piggott-Solo (linear Hawkes, least squares, multiplicative non-negative update, no theorem, stability not enforced), Pasha-Solo (log-linear model, likelihood steepest ascent, heuristic averaging, unproved PD of E[phi phi' lambda]) and Spreij 1986/1991 now read in full; paragraphs corrected in literature_difference_statements.md. Main consequence: Spreij anticipates the well-specified recursion and its CLT.</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2106,7 @@
       </c>
       <c r="M24" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. literature_unverified_items.md. Searched/fetched all listed items. Zhang 2023: no matching paper found (identity unresolved). Wang 2023 = Technometrics online CUSUM change-point detector (not an estimator). Online EM for Hawkes: none found; Zhou-Zha-Song is batch ADMM; Lemonnier-Vayatis attribution unconfirmed. Cartea-Cohen-Labyad: batch LS gradient sampling, no regret. Bacry et al.: no misspecification paper located. Citation trees screened by titles (Hall-Willett via Semantic Scholar: 64; Yang et al. via OpenAlex: 26; a second Semantic Scholar query hit HTTP 429). Found beyond the list: Wei-Zhu-Zhang-Xie AISTATS 2021 (KL pseudo-truth, QMLE sandwich), Rong-Nair 2026 (LS pseudo-truth, CLT), Spreij 1986/1991 (recursive estimators for counting processes), Pasha-Solo CDC 2019 (fixed-gain), Lima 2021 (eps-margin stabilisation). Overlap-risk column updated. UNRESOLVED: Zhang 2023, online EM, full texts of Spreij/Solo papers.</t>
+          <t> 25 Oct 2026. literature_unverified_items.md. Searched/fetched all listed items. Zhang 2023: no matching paper found (identity unresolved). Wang 2023 = Technometrics online CUSUM change-point detector (not an estimator). Online EM for Hawkes: none found; Zhou-Zha-Song is batch ADMM; Lemonnier-Vayatis attribution unconfirmed. Cartea-Cohen-Labyad: batch LS gradient sampling, no regret. Bacry et al.: no misspecification paper located. Citation trees screened by titles (Hall-Willett via Semantic Scholar: 64; Yang et al. via OpenAlex: 26; a second Semantic Scholar query hit HTTP 429). Found beyond the list: Wei-Zhu-Zhang-Xie AISTATS 2021 (KL pseudo-truth, QMLE sandwich), Rong-Nair 2026 (LS pseudo-truth, CLT), Spreij 1986/1991 (recursive estimators for counting processes), Pasha-Solo CDC 2019 (fixed-gain), Lima 2021 (eps-margin stabilisation). Overlap-risk column updated. UNRESOLVED: Zhang 2023, online EM, full texts of Spreij/Solo papers. UPDATE 25 Oct 2026: Spreij 1986/1991, Piggott-Solo 2018 and Pasha-Solo 2019 read in full (refpapers_conclusions.md). Spreij confirmed as the key prior art for Problem 17 (well-specified part); the Solo papers have no theorems.</t>
         </is>
       </c>
     </row>
@@ -3763,12 +3767,12 @@
       </c>
       <c r="G7" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H7" s="32" t="inlineStr">
         <is>
-          <t>Reading: abstract read 25 Oct 2026 (via OpenAlex); full text NOT obtained. Fixed-gain exponentially weighted least squares on a Laguerre basis, non-negativity preserving, two time scales, simulations; abstract states no regret bound or near-critical analysis. See literature_search_report.md. Also: Pasha and Solo, CDC 2019, Adaptive Estimation of a Vector Point Process Model (abstract: fixed-gain adaptive estimator on the instantaneous likelihood, non-negativity constraints, genomic application). Full texts of both still not obtained.</t>
+          <t>READ IN FULL 25 Oct 2026. Linear Hawkes, Laguerre basis (one shared decay constant), exponentially weighted LEAST SQUARES via a one-step NMF multiplicative update, fixed gain, discrete bins; simulations only; stability not enforced; no theorem. Claims projections can stall. Pasha-Solo (CDC 2019) read in full too: log-linear model, likelihood steepest ascent, heuristic averaging analysis assuming well-specification. See refpapers_conclusions.md.</t>
         </is>
       </c>
     </row>
@@ -4740,7 +4744,7 @@
       </c>
       <c r="H31" s="32" t="inlineStr">
         <is>
-          <t>Abstract-level only (25 Oct 2026); the scans are image-only and were not OCRed. Likely anticipates the well-specified recursive consistency/CLT of Problem 17; misspecification, active constraint, regret, near-critical not known to be covered. Read first.</t>
+          <t>READ IN FULL 25 Oct 2026 (both papers; equations from page images). Intensity lambda=theta'phi with observed predictable phi, well-specified. AML recursion = our EF Newton in continuous time; 1986 Thm 3.2 and 1991 Thm 3 give a.s. consistency (Lyapunov x'Q^-1 x; Lai-Wei growth; known box [eps,1/eps]); 1986 Thm 5.4 / 1991 Thm 7 give the Cramer-Rao CLT. No Hawkes example, misspecification, regret, near-critical. Anticipates the well-specified parts of Thms 17A/17B and the algorithm of Problem 5. See refpapers_conclusions.md.</t>
         </is>
       </c>
     </row>
@@ -4777,12 +4781,12 @@
       </c>
       <c r="G32" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H32" s="32" t="inlineStr">
         <is>
-          <t>Abstract only (25 Oct 2026). Companion of the Piggott-Solo row.</t>
+          <t>READ IN FULL 25 Oct 2026. Log-linear (nonlinear) Hawkes, no sign constraints, fixed-gain likelihood steepest ascent, heuristic averaging stability sketch (stationary, well-specified; PD of E[phi phi' lambda] and the hovering theorem left unproved). Not the linear model of this project; no theorem on misspecification, regret or tracking.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
LaTeX integration: add Section 'epsilon-dependence' and 'numerical validation' (Problems 6, 8, 9, 19-21) next to the misspecification part (Problems 16-18); update review (concordance, errata, status matrix, open problems), master (graphicx, abstract), checker; add notes, code and literature records for Problems 16-18
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hawkes_research_problem_tracker.xlsx
+++ b/hawkes_research_problem_tracker.xlsx
@@ -1687,7 +1687,7 @@
       </c>
       <c r="M17" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. problem16_kl_pseudotruth.md; code/p16/ (sim16.c, p16lib.py, t1..t7.py). Theorem 16 [P, draft, not independently verified]: under finite rate and E[lam*(1+|a|^2)]&lt;inf, L(theta)=E[lam* log(lam*/lam_theta)-lam*+lam_theta] is convex, strictly convex for distinct beta_k (linear independence of exponentials on a gap), coercive on the cone, so a unique theta-dagger exists on Theta_eps and on the cone; KKT: dL/dmu=E[1-lam*/lam]=rho_0, dL/dalpha_k=E[S_k(1-lam*/lam)]=rho_k-kappa/beta_k. Rate matching (new): mu-dagger=(1-n-dagger)Lambda* minus multiplier terms, so n(theta-dagger)&lt;1 automatically and the constraint n&lt;=1-eps is active iff the unconstrained immigrant share mu/Lambda* &lt; eps; when active mu-dagger=eps*Lambda*-kappa(1-eps). Quasi-MLE converges a.s. to theta-dagger. Numerics (power-law truth n*=0.8,0.95, K=1..4): rate matching to 4 digits, unique minimiser from several starts, KKT/kappa identities hold under active constraint, error of QMLE ~T^-1/2, Newton-decrement bound never violated. Found: n(theta-dagger)&lt;n*, increasing with K (0.46,0.62,0.70,0.73 at n*=0.8) - input to Problem 18. KL and quadratic surrogate differ by only 0.1-0.3% in these examples, so the advantage is structural not numerical. NOT proved: explicit strong-convexity constant, sandwich variance, a priori mu-dagger&gt;mu_min. SECOND PASS 25 Oct 2026 (problem16_kl_pseudotruth.md sec. 8, code/p16/t8.py, t9.py): explicit strong-convexity constant Hess L &gt;= lam_lo*E[aa'/(Lambda*+sum beta_k S_k)^2] (certified, valid and non-vacuous in all runs, conservative by 17-300x, worse with K and n*); consistency of the QMLE written out; sandwich variance H^-1 J H^-1 with J=H+misspecification terms, reproduced numerically (naive H^-1/T underestimates var(mu) by 40%, sandwich by 17%; equal in the well-specified control); CLT tagged P* (needs mixing). Still open: an a priori proof that mu-dagger&gt;mu_min (the natural bounds are vacuous; only the a-posteriori convexity certificate holds), active-constraint limit law. Replaces the earlier 'NOT proved' list except those two items. THIRD PASS 25 Oct 2026 (sec. 9, code/p16/t10.py, t11.py, t12.py): closed the last two open items. (i) A priori lower bound mu-dagger &gt;= mu_0, mu_0 = sup{mu: min_{alpha in A_eps} E[lam*/(mu+alpha'S)] &gt;= 1} [P], computable from the data law alone; non-vacuous in all runs (Phi(0)=1.06-1.63) but conservative 2-7x (mu_0~0.28 vs mu-dagger 1.55 at K=3, eps=0.05). (ii) Limit law with active constraints [P*]: sqrt(T)(theta-hat - theta-dagger) -&gt; V(V'HV)^-1 V'Z, rank d-|active|; tested K=2, n&lt;=0.5 active: var(mu) 3.41e-3 empirical vs 3.45e-3 formula (population J), corr -0.209 vs -0.210; unconstrained sandwich overstates 5x. Remaining caveats: CLT needs mixing (P*), strict complementarity assumed, batch-means J is 17-27% low at B=20.</t>
+          <t> 25 Oct 2026. problem16_kl_pseudotruth.md; code/p16/ (sim16.c, p16lib.py, t1..t7.py). Theorem 16 [P, draft, not independently verified]: under finite rate and E[lam*(1+|a|^2)]&lt;inf, L(theta)=E[lam* log(lam*/lam_theta)-lam*+lam_theta] is convex, strictly convex for distinct beta_k (linear independence of exponentials on a gap), coercive on the cone, so a unique theta-dagger exists on Theta_eps and on the cone; KKT: dL/dmu=E[1-lam*/lam]=rho_0, dL/dalpha_k=E[S_k(1-lam*/lam)]=rho_k-kappa/beta_k. Rate matching (new): mu-dagger=(1-n-dagger)Lambda* minus multiplier terms, so n(theta-dagger)&lt;1 automatically and the constraint n&lt;=1-eps is active iff the unconstrained immigrant share mu/Lambda* &lt; eps; when active mu-dagger=eps*Lambda*-kappa(1-eps). Quasi-MLE converges a.s. to theta-dagger. Numerics (power-law truth n*=0.8,0.95, K=1..4): rate matching to 4 digits, unique minimiser from several starts, KKT/kappa identities hold under active constraint, error of QMLE ~T^-1/2, Newton-decrement bound never violated. Found: n(theta-dagger)&lt;n*, increasing with K (0.46,0.62,0.70,0.73 at n*=0.8) - input to Problem 18. KL and quadratic surrogate differ by only 0.1-0.3% in these examples, so the advantage is structural not numerical. NOT proved: explicit strong-convexity constant, sandwich variance, a priori mu-dagger&gt;mu_min. SECOND PASS 25 Oct 2026 (problem16_kl_pseudotruth.md sec. 8, code/p16/t8.py, t9.py): explicit strong-convexity constant Hess L &gt;= lam_lo*E[aa'/(Lambda*+sum beta_k S_k)^2] (certified, valid and non-vacuous in all runs, conservative by 17-300x, worse with K and n*); consistency of the QMLE written out; sandwich variance H^-1 J H^-1 with J=H+misspecification terms, reproduced numerically (naive H^-1/T underestimates var(mu) by 40%, sandwich by 17%; equal in the well-specified control); CLT tagged P* (needs mixing). Still open: an a priori proof that mu-dagger&gt;mu_min (the natural bounds are vacuous; only the a-posteriori convexity certificate holds), active-constraint limit law. Replaces the earlier 'NOT proved' list except those two items. THIRD PASS 25 Oct 2026 (sec. 9, code/p16/t10.py, t11.py, t12.py): closed the last two open items. (i) A priori lower bound mu-dagger &gt;= mu_0, mu_0 = sup{mu: min_{alpha in A_eps} E[lam*/(mu+alpha'S)] &gt;= 1} [P], computable from the data law alone; non-vacuous in all runs (Phi(0)=1.06-1.63) but conservative 2-7x (mu_0~0.28 vs mu-dagger 1.55 at K=3, eps=0.05). (ii) Limit law with active constraints [P*]: sqrt(T)(theta-hat - theta-dagger) -&gt; V(V'HV)^-1 V'Z, rank d-|active|; tested K=2, n&lt;=0.5 active: var(mu) 3.41e-3 empirical vs 3.45e-3 formula (population J), corr -0.209 vs -0.210; unconstrained sandwich overstates 5x. Remaining caveats: CLT needs mixing (P*), strict complementarity assumed, batch-means J is 17-27% low at B=20. NOVELTY CORRECTION 25 Oct 2026 (Rong-Nair PDF checked): the surrogate (least-squares) rate matching c* = Lambda(1-Gamma*) and the spectral form of the LS pseudo-truth are KNOWN (their Lemma 4(b), Lemma 13, Thm 15, eq. 5.7). Ours: the KL rate matching and n-dagger&lt;1 (their Gamma*&lt;1 is unproved), binding criterion, active-constraint limit law, strong-convexity constant. Their CLT-without-mixing uses a linear martingale representation of lambda via the Hawkes resolvent and does not transfer to the KL score, so the mixing caveat stays.</t>
         </is>
       </c>
     </row>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="M18" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. problem17_online_convergence.md; code/p17/ (online17.c, lib17.py, w1,m1,m2,m3,trap,ev). Draft, not independently verified. Theorem 17A [P*]: projected online Newton (Fisher or observed-information preconditioner, exact F-norm projection) converges a.s. to the unique constrained KL pseudo-truth theta-dagger_Theta of Problem 16, active constraint included (ODE method with Markov noise + matrix gain; relies on cited Benveniste-Metivier-Priouret conditions, not re-verified). New exact facts: Lyapunov drift of ||theta-theta-dagger||^2_F is -v'(2Hbar - I_F)v with a favourable-sign multiplier term when the constraint binds; A = I_F^-1 H has eigenvalue exactly 1 at an interior theta-dagger. Theorem 17B/C [P*]: sqrt(n)(theta_n - theta-dagger) -&gt; N(0,Sigma), Lyapunov equation (A-1/2)Sigma+Sigma(A-1/2)'=Lambda* Ibar^-1 J Ibar^-1; with observed-information preconditioner Sigma = Lambda* H^-1 J H^-1 (batch sandwich) with no side condition; active constraint: same in the face subspace, n*dist to face -&gt; const (O(1/n)), projection active in a stable 3% of steps. Numerics (power-law truth n*=0.8, K=2, 600 replicates up to 1e5 events): n*Var matches prediction to 5-14% interior and 1-12% with active constraint (MC ~6%); n*MSE flat (rate 1/n); eigenvalues of I_F^-1 H in [0.97,1.002] in every example so EF=OI; OI corner-trapping found in 1/300 runs when mu_min=1e-3, none for EF or mu_min&gt;=0.1. MISSING for Done: self-contained proof of the Poisson-equation/regularity step, rigorous excursion bound for the distance to the face, degenerate (no strict complementarity) case, regret statement (Prop 17.4 is a conjecture), K&gt;2. READ 25 Oct 2026 (refpapers_conclusions.md): the EF recursion is Spreij's AML recursion (Stochastics 1986; JMVA 1991) applied to the Hawkes regressor; his well-specified a.s. consistency (Lyapunov x'Q^-1 x, Lai-Wei growth condition, known coordinate box) and Cramer-Rao CLT are the A=I special case of Theorems 17A/17B, which are therefore NOT claimed as new. Still ours: misspecified target theta-dagger, drift matrix I_F^-1 H != I and the Lyapunov-equation limit law (+ Lemma 17.5), observed-information preconditioner, exact convex projection with a binding stability face / alpha_k=0, active-constraint limit law, regret. Overlap risk: High for the well-specified part, Low-Medium for the rest.</t>
+          <t> 25 Oct 2026. problem17_online_convergence.md; code/p17/ (online17.c, lib17.py, w1,m1,m2,m3,trap,ev). Draft, not independently verified. Theorem 17A [P*]: projected online Newton (Fisher or observed-information preconditioner, exact F-norm projection) converges a.s. to the unique constrained KL pseudo-truth theta-dagger_Theta of Problem 16, active constraint included (ODE method with Markov noise + matrix gain; relies on cited Benveniste-Metivier-Priouret conditions, not re-verified). New exact facts: Lyapunov drift of ||theta-theta-dagger||^2_F is -v'(2Hbar - I_F)v with a favourable-sign multiplier term when the constraint binds; A = I_F^-1 H has eigenvalue exactly 1 at an interior theta-dagger. Theorem 17B/C [P*]: sqrt(n)(theta_n - theta-dagger) -&gt; N(0,Sigma), Lyapunov equation (A-1/2)Sigma+Sigma(A-1/2)'=Lambda* Ibar^-1 J Ibar^-1; with observed-information preconditioner Sigma = Lambda* H^-1 J H^-1 (batch sandwich) with no side condition; active constraint: same in the face subspace, n*dist to face -&gt; const (O(1/n)), projection active in a stable 3% of steps. Numerics (power-law truth n*=0.8, K=2, 600 replicates up to 1e5 events): n*Var matches prediction to 5-14% interior and 1-12% with active constraint (MC ~6%); n*MSE flat (rate 1/n); eigenvalues of I_F^-1 H in [0.97,1.002] in every example so EF=OI; OI corner-trapping found in 1/300 runs when mu_min=1e-3, none for EF or mu_min&gt;=0.1. MISSING for Done: self-contained proof of the Poisson-equation/regularity step, rigorous excursion bound for the distance to the face, degenerate (no strict complementarity) case, regret statement (Prop 17.4 is a conjecture), K&gt;2. READ 25 Oct 2026 (refpapers_conclusions.md): the EF recursion is Spreij's AML recursion (Stochastics 1986; JMVA 1991) applied to the Hawkes regressor; his well-specified a.s. consistency (Lyapunov x'Q^-1 x, Lai-Wei growth condition, known coordinate box) and Cramer-Rao CLT are the A=I special case of Theorems 17A/17B, which are therefore NOT claimed as new. Still ours: misspecified target theta-dagger, drift matrix I_F^-1 H != I and the Lyapunov-equation limit law (+ Lemma 17.5), observed-information preconditioner, exact convex projection with a binding stability face / alpha_k=0, active-constraint limit law, regret. Overlap risk: High for the well-specified part, Low-Medium for the rest. SPREIJ COROLLARY 25 Oct 2026 (refpapers_conclusions.md 5.2): Spreij 1991 Thm 3 applies to the Hawkes dictionary (conditions verified: G_t/t -&gt; positive definite limit by the ergodic theorem and Wasserstein contraction; f(x)=x^2 growth condition holds), so the well-specified AML recursion is a.s. consistent at every fixed n&lt;1 without the Problem 5 concentration machinery (no rate/regret/eps-explicit constants). Numerics code/p17/spreij_cond.py: transient lengthens as eps falls (condition number of G_t ~3e4 at n=0.97). SELF-CONTAINED PROOF 25 Oct 2026 (problem17 section 7, code/p17/t_drift.py, t_kappa.py): Theorem 17A* [P]: a.s. convergence of the EF/OI recursion with gain constant kappa to the constrained KL pseudo-truth WITHOUT citing stochastic-approximation theory, under the drift condition (D_kappa) E[kappa (v'a)^2/lam_theta] - 2 v'grad L(theta) &lt;= 0 on Theta. Proof: F-norm Lyapunov function + non-expansive projection; every non-drift term is o(t) by the ergodic theorem / martingale SLLN (no Poisson equation, no rates, no Markov property of the truth); W_N=o(N) and W_N&gt;=cN|v|^2 give v-&gt;0. Closed form: Psi-bar = -2v'gradL(theta-dagger) - E[(v'a)^2 (2 lam* - kappa lam-dagger)/(lam-dagger lam_theta)], so (D_kappa) holds for kappa&lt;=2 inf lam*/lam-dagger (EF) and, for OI, on a ratio-restricted Theta; well-specified: all kappa&lt;=2. Numerics: D_1 holds on random samples of Theta for EF (K=1 strong misspec, K=2, active constraint; max Psi-bar/|v|^2 = -0.027,-0.016,-0.026), fails at kappa=2 and, for OI, at extreme theta; all kappa (0.5-4) converge numerically (condition is sufficient, not necessary). Still open: general result without D_kappa (cited ODE route), rates, regret.</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="M19" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026. problem18_bias_vs_K.md; code/p18/ (fd18.py, e2..e8.py). Draft, not independently verified. PROVED reductions: (i) n*-n-dagger = (mu-dagger - mu*)/Lambda* (rate matching, Problem 16); (ii) the surrogate pseudo-truth is the weighted L2 pole approximant of G(s)=int nu/(beta+s) on the imaginary axis with weight Lambda*/|1-G|^2 (Hawkes spectrum), so the bias is the DC value of the approximation error and can be computed deterministically for any K (matches the simulations of Problem 16 to 0.004). CONJECTURE 18.4 (numerically supported): b_K = kappa(eta,r) * n* (tau beta_1)^eta / Gamma(1+eta), beta_1 = beta_top r^-(K-1), i.e. geometric decay in K at rate eta*ln r; kappa ~0.43 at eta=1/2 (0.7 at eta=0.15), independent of n* and of criticality; exponent confirmed over 3 decades of beta_1 (ratios 0.32 per decade vs 10^-0.5); fixed range saturates at the truncation floor kappa*n_low(beta_min). Also: coarse grids overshoot (bias changes sign; best ratio for fixed K: r~17 at K=4, 8 at K=6, 6 at K=8); KL and surrogate biases agree within ~0.002 for K&gt;=3. NOT proved: the exponent eta and kappa&gt;0 (Wiener-Hopf/Newman-Stahl type problem for a geometric pole ladder), the discretization-floor law ~exp(-pi^2/ln r), general nu beyond the gamma form.</t>
+          <t> 25 Oct 2026. problem18_bias_vs_K.md; code/p18/ (fd18.py, e2..e8.py). Draft, not independently verified. PROVED reductions: (i) n*-n-dagger = (mu-dagger - mu*)/Lambda* (rate matching, Problem 16); (ii) the surrogate pseudo-truth is the weighted L2 pole approximant of G(s)=int nu/(beta+s) on the imaginary axis with weight Lambda*/|1-G|^2 (Hawkes spectrum), so the bias is the DC value of the approximation error and can be computed deterministically for any K (matches the simulations of Problem 16 to 0.004). CONJECTURE 18.4 (numerically supported): b_K = kappa(eta,r) * n* (tau beta_1)^eta / Gamma(1+eta), beta_1 = beta_top r^-(K-1), i.e. geometric decay in K at rate eta*ln r; kappa ~0.43 at eta=1/2 (0.7 at eta=0.15), independent of n* and of criticality; exponent confirmed over 3 decades of beta_1 (ratios 0.32 per decade vs 10^-0.5); fixed range saturates at the truncation floor kappa*n_low(beta_min). Also: coarse grids overshoot (bias changes sign; best ratio for fixed K: r~17 at K=4, 8 at K=6, 6 at K=8); KL and surrogate biases agree within ~0.002 for K&gt;=3. NOT proved: the exponent eta and kappa&gt;0 (Wiener-Hopf/Newman-Stahl type problem for a geometric pole ladder), the discretization-floor law ~exp(-pi^2/ln r), general nu beyond the gamma form. NOVELTY CORRECTION 25 Oct 2026: Prop 18.2 (frequency-domain weighted-L2 form with the Hawkes Bartlett spectrum) is KNOWN for least squares: Rong-Nair arXiv 2602.20795 Lemma 4(b), Lemma 13(b), Thm 15. Not claimed. The bias law in K for a power-law truth (Conjecture 18.4) is not in their paper (their numerics: sum-of-exponentials truth, Laguerre P=1..5, non-monotone, no rate).</t>
         </is>
       </c>
     </row>
@@ -1987,12 +1987,12 @@
       </c>
       <c r="L22" s="32" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="M22" s="33" t="inlineStr">
         <is>
-          <t> 25 Oct 2026, problem21_baselines.md; code/p21_baselines.cs, p21_run.sh, p21_analyze.py, p21_summary.txt; figures/p21_*.png. SIMULATED HALF DONE: batch MLE (constrained, same box), Hall-Willett-type mirror descent (log mirror map on theta, const / 1/sqrt(i) / 1/i steps, 6 step sizes) and Solo-type fixed-gain EWLS (rho = 1, 1-1/2000, 1-1/200), all on identical paths (K=1 eps 0.3/0.1/0.03, K=2 eps 0.1), error + regret + CPU. RESULTS at n=1e5: ours e_n = batch MLE to 0.01-0.02 (1.78/1.80, 2.16/2.15, 1.86/1.87, K=2 4.08/4.09; target d); ours better than batch at small n (n=95: 0.83 vs 4.50). Solo-type rho=1 inefficient by the predicted factor tr(I B^-1 C B^-1)/d = 1.22/1.50/1.75/1.38 (predicted 2.45/2.99/3.50/4.15, measured 2.48/3.66/3.08/4.92), fixed gain has non-vanishing error (e_n ~ n, linear regret). HW-type with eta0 tuned on the truth is 4.5-28x above d (no curvature, condition number ~ eps^-2); default step diverges. COST: ours 1.6 us/event (K=1), 2.3 (K=2), constant; mirror descent 0.08/0.10; EWLS 0.42/0.59; batch refit 0.33-0.4 us per data event per refit (linear in n), keeping batch current after every event ~ 1.1-1.3e4 us/event at n=2e5 (6000-7000x ours). CAVEATS: HW and Solo are adaptations (HW designed for intensity tracking with sqrt T regret, Solo read as abstract only; fixed gain is a feature for tracking, not static estimation). MISSING for Done: real-data comparison (needs tick data, Problem 20); protocol fixed (same stream, same box, distance to full-sample MLE and held-out log-loss replace e_n).</t>
+          <t> 25 Oct 2026, problem21_baselines.md; code/p21_baselines.cs, p21_run.sh, p21_analyze.py, p21_summary.txt; figures/p21_*.png. SIMULATED HALF DONE: batch MLE (constrained, same box), Hall-Willett-type mirror descent (log mirror map on theta, const / 1/sqrt(i) / 1/i steps, 6 step sizes) and Solo-type fixed-gain EWLS (rho = 1, 1-1/2000, 1-1/200), all on identical paths (K=1 eps 0.3/0.1/0.03, K=2 eps 0.1), error + regret + CPU. RESULTS at n=1e5: ours e_n = batch MLE to 0.01-0.02 (1.78/1.80, 2.16/2.15, 1.86/1.87, K=2 4.08/4.09; target d); ours better than batch at small n (n=95: 0.83 vs 4.50). Solo-type rho=1 inefficient by the predicted factor tr(I B^-1 C B^-1)/d = 1.22/1.50/1.75/1.38 (predicted 2.45/2.99/3.50/4.15, measured 2.48/3.66/3.08/4.92), fixed gain has non-vanishing error (e_n ~ n, linear regret). HW-type with eta0 tuned on the truth is 4.5-28x above d (no curvature, condition number ~ eps^-2); default step diverges. COST: ours 1.6 us/event (K=1), 2.3 (K=2), constant; mirror descent 0.08/0.10; EWLS 0.42/0.59; batch refit 0.33-0.4 us per data event per refit (linear in n), keeping batch current after every event ~ 1.1-1.3e4 us/event at n=2e5 (6000-7000x ours). CAVEATS: HW and Solo are adaptations (HW designed for intensity tracking with sqrt T regret, Solo read as abstract only; fixed gain is a feature for tracking, not static estimation). MISSING for Done: real-data comparison (needs tick data, Problem 20); protocol fixed (same stream, same box, distance to full-sample MLE and held-out log-loss replace e_n). 25 Oct 2026 (real-data half), problem21_baselines.md sections 7-8; code/p21_real.cs, p21_real_analyze.py, p21_real_summary.txt; figures/p21_real.png. REAL STREAM (Deribit BTC option trades, 1.74M events, 365 daily windows, K=3): prequential log-loss regret vs best fixed theta in hindsight on days 60-364, every family's hyperparameter chosen on days 0-59 with bracketed grids. Results (1e-3 nats/event; negative = beats any fixed theta): ours forgetting m=0.05 -35.8 (best without test-period info; also beats the per-day oracle -22.6), HW-type eta0/sqrt(i) -19.5, Solo-type EWLS rho=1-1/100 -8.5, batch 30-day -2.4, ours growing +1.2 = batch all-history +1.4 (equal), HW eta0/i +20.6, HW constant-step chosen on dev diverges +215 (test-tuned constant step -37.7 ties ours but is stable only for eta0&lt;=0.03; ours stable over m in [0.02,20]). Distance to pooled batch MLE: growing Newton 1.6/1.2/6.0/22.8 at days 5/30/120/364 (chi2_4 scale), forgetting/fixed-gain 1e3-1e5 (not an accuracy criterion on a non-stationary stream). CPU: ours 4.98 us/event, EWLS 0.71, HW 0.097, batch daily refit 281 us/event amortised (56x ours). CAVEATS: BTC not NSE; HW/Solo adaptations; one stream/dictionary/split.</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="H8" s="32" t="inlineStr">
         <is>
-          <t>Read 25 Oct 2026 (first ~200k of 213k characters of the HTML). Batch LS on a prescribed unit-mass basis; pseudo-true parameters via the LS contrast (Section 5.3, Thm 15) and CLTs under correct spec (Thm 17) and misspecification (Thm 21) by a martingale route with no mixing; numerics P=1..5 vs a sum-of-exponentials truth (no rate, no power law). No KL, no online, no proof of Gamma*&lt;1. May anticipate Prop 18.2 and the surrogate rate matching; route for the CLT item. See literature_difference_statements.md.</t>
+          <t>Read 25 Oct 2026 (first ~200k of 213k characters of the HTML). Batch LS on a prescribed unit-mass basis; pseudo-true parameters via the LS contrast (Section 5.3, Thm 15) and CLTs under correct spec (Thm 17) and misspecification (Thm 21) by a martingale route with no mixing; numerics P=1..5 vs a sum-of-exponentials truth (no rate, no power law). No KL, no online, no proof of Gamma*&lt;1. May anticipate Prop 18.2 and the surrogate rate matching; route for the CLT item. See literature_difference_statements.md. CHECKED 25 Oct 2026 in the PDF: Lemma 4(b) Bartlett spectrum Lambda/|1-phi0^|^2; Lemma 13 and eq. (5.2)-(5.5) spectral integrals for R*, R*^(1,0); Thm 15 alpha*=R*^-1 R*^(1,0), c*=Lambda(1-Gamma*). So the spectral weighted-L2 form of the LS pseudo-truth and the surrogate rate matching are known; Gamma*&lt;1 not proved; CLT without mixing relies on the linear resolvent martingale representation (no transfer to the KL score).</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="H30" s="32" t="inlineStr">
         <is>
-          <t>Read 25 Oct 2026 (about 100k of 136k characters of ar5iv). Piecewise-constant triggering, batch, near-critical not analysed. Anticipates the generic part of Theorem 16 / Prop 16.7; not the exponential dictionary with stability set, rate matching, active constraint, online.</t>
+          <t>Read 25 Oct 2026 (about 100k of 136k characters of ar5iv). Piecewise-constant triggering, batch, near-critical not analysed. Anticipates the generic part of Theorem 16 / Prop 16.7; not the exponential dictionary with stability set, rate matching, active constraint, online. Further 25 Oct 2026: consistency and CLT are taken from modifications of Ogata (1978) Thms 2, 4, 5; only equality constraints appear (no KKT/inequality constraints); the piecewise-constant model is linear in the bin heights (same linear-in-parameter structure as ours). Proof of Lemma 1 itself not retrieved.</t>
         </is>
       </c>
     </row>

</xml_diff>